<commit_message>
자동 수집: 2026-07-15 07:13 UTC
</commit_message>
<xml_diff>
--- a/reports/부정리뷰리포트_20260715.xlsx
+++ b/reports/부정리뷰리포트_20260715.xlsx
@@ -20,14 +20,14 @@
     <sheet name="IOS글로벌" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'안드로이드개인'!$A$5:$D$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'안드로이드개인'!$A$5:$D$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'IOS개인'!$A$5:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'안드로이드기업'!$A$5:$D$118</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'IOS기업'!$A$5:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'안드로이드알림'!$A$5:$D$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'IOS알림'!$A$5:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'안드로이드미니'!$A$5:$D$141</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'IOS미니'!$A$5:$D$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'IOS미니'!$A$5:$D$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'안드로이드글로벌'!$A$5:$D$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'IOS글로벌'!$A$5:$D$6</definedName>
   </definedNames>
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L387"/>
+  <dimension ref="A1:L353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1325,7 +1325,7 @@
         </is>
       </c>
       <c r="B37" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C37" s="4" t="inlineStr"/>
       <c r="D37" s="4" t="inlineStr"/>
@@ -1337,7 +1337,7 @@
       <c r="J37" s="4" t="inlineStr"/>
       <c r="K37" s="4" t="inlineStr"/>
       <c r="L37" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -5129,13 +5129,11 @@
       </c>
       <c r="G209" s="4" t="inlineStr"/>
       <c r="H209" s="4" t="inlineStr"/>
-      <c r="I209" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I209" s="4" t="inlineStr"/>
       <c r="J209" s="4" t="inlineStr"/>
       <c r="K209" s="4" t="inlineStr"/>
       <c r="L209" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210">
@@ -5537,7 +5535,7 @@
     <row r="228">
       <c r="A228" s="4" t="inlineStr">
         <is>
-          <t>01월 03일</t>
+          <t>12월 09일</t>
         </is>
       </c>
       <c r="B228" s="4" t="inlineStr"/>
@@ -5546,10 +5544,10 @@
       <c r="E228" s="4" t="inlineStr"/>
       <c r="F228" s="4" t="inlineStr"/>
       <c r="G228" s="4" t="inlineStr"/>
-      <c r="H228" s="4" t="inlineStr"/>
-      <c r="I228" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H228" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I228" s="4" t="inlineStr"/>
       <c r="J228" s="4" t="inlineStr"/>
       <c r="K228" s="4" t="inlineStr"/>
       <c r="L228" s="5" t="n">
@@ -5559,7 +5557,7 @@
     <row r="229">
       <c r="A229" s="4" t="inlineStr">
         <is>
-          <t>12월 09일</t>
+          <t>12월 06일</t>
         </is>
       </c>
       <c r="B229" s="4" t="inlineStr"/>
@@ -5568,11 +5566,11 @@
       <c r="E229" s="4" t="inlineStr"/>
       <c r="F229" s="4" t="inlineStr"/>
       <c r="G229" s="4" t="inlineStr"/>
-      <c r="H229" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H229" s="4" t="inlineStr"/>
       <c r="I229" s="4" t="inlineStr"/>
-      <c r="J229" s="4" t="inlineStr"/>
+      <c r="J229" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K229" s="4" t="inlineStr"/>
       <c r="L229" s="5" t="n">
         <v>1</v>
@@ -5581,7 +5579,7 @@
     <row r="230">
       <c r="A230" s="4" t="inlineStr">
         <is>
-          <t>12월 06일</t>
+          <t>12월 05일</t>
         </is>
       </c>
       <c r="B230" s="4" t="inlineStr"/>
@@ -5590,22 +5588,20 @@
       <c r="E230" s="4" t="inlineStr"/>
       <c r="F230" s="4" t="inlineStr"/>
       <c r="G230" s="4" t="inlineStr"/>
-      <c r="H230" s="4" t="inlineStr"/>
-      <c r="I230" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J230" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H230" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I230" s="4" t="inlineStr"/>
+      <c r="J230" s="4" t="inlineStr"/>
       <c r="K230" s="4" t="inlineStr"/>
       <c r="L230" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="4" t="inlineStr">
         <is>
-          <t>12월 05일</t>
+          <t>10월 11일</t>
         </is>
       </c>
       <c r="B231" s="4" t="inlineStr"/>
@@ -5627,7 +5623,7 @@
     <row r="232">
       <c r="A232" s="4" t="inlineStr">
         <is>
-          <t>11월 30일</t>
+          <t>07월 24일</t>
         </is>
       </c>
       <c r="B232" s="4" t="inlineStr"/>
@@ -5636,20 +5632,20 @@
       <c r="E232" s="4" t="inlineStr"/>
       <c r="F232" s="4" t="inlineStr"/>
       <c r="G232" s="4" t="inlineStr"/>
-      <c r="H232" s="4" t="inlineStr"/>
-      <c r="I232" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="H232" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I232" s="4" t="inlineStr"/>
       <c r="J232" s="4" t="inlineStr"/>
       <c r="K232" s="4" t="inlineStr"/>
       <c r="L232" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="4" t="inlineStr">
         <is>
-          <t>10월 11일</t>
+          <t>05월 12일</t>
         </is>
       </c>
       <c r="B233" s="4" t="inlineStr"/>
@@ -5658,11 +5654,11 @@
       <c r="E233" s="4" t="inlineStr"/>
       <c r="F233" s="4" t="inlineStr"/>
       <c r="G233" s="4" t="inlineStr"/>
-      <c r="H233" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H233" s="4" t="inlineStr"/>
       <c r="I233" s="4" t="inlineStr"/>
-      <c r="J233" s="4" t="inlineStr"/>
+      <c r="J233" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K233" s="4" t="inlineStr"/>
       <c r="L233" s="5" t="n">
         <v>1</v>
@@ -5671,7 +5667,7 @@
     <row r="234">
       <c r="A234" s="4" t="inlineStr">
         <is>
-          <t>07월 24일</t>
+          <t>04월 08일</t>
         </is>
       </c>
       <c r="B234" s="4" t="inlineStr"/>
@@ -5681,19 +5677,19 @@
       <c r="F234" s="4" t="inlineStr"/>
       <c r="G234" s="4" t="inlineStr"/>
       <c r="H234" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I234" s="4" t="inlineStr"/>
       <c r="J234" s="4" t="inlineStr"/>
       <c r="K234" s="4" t="inlineStr"/>
       <c r="L234" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="4" t="inlineStr">
         <is>
-          <t>05월 12일</t>
+          <t>02월 19일</t>
         </is>
       </c>
       <c r="B235" s="4" t="inlineStr"/>
@@ -5703,21 +5699,19 @@
       <c r="F235" s="4" t="inlineStr"/>
       <c r="G235" s="4" t="inlineStr"/>
       <c r="H235" s="4" t="inlineStr"/>
-      <c r="I235" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I235" s="4" t="inlineStr"/>
       <c r="J235" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K235" s="4" t="inlineStr"/>
       <c r="L235" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="4" t="inlineStr">
         <is>
-          <t>04월 08일</t>
+          <t>02월 08일</t>
         </is>
       </c>
       <c r="B236" s="4" t="inlineStr"/>
@@ -5727,19 +5721,19 @@
       <c r="F236" s="4" t="inlineStr"/>
       <c r="G236" s="4" t="inlineStr"/>
       <c r="H236" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I236" s="4" t="inlineStr"/>
       <c r="J236" s="4" t="inlineStr"/>
       <c r="K236" s="4" t="inlineStr"/>
       <c r="L236" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="4" t="inlineStr">
         <is>
-          <t>02월 19일</t>
+          <t>01월 26일</t>
         </is>
       </c>
       <c r="B237" s="4" t="inlineStr"/>
@@ -5761,7 +5755,7 @@
     <row r="238">
       <c r="A238" s="4" t="inlineStr">
         <is>
-          <t>02월 08일</t>
+          <t>01월 15일</t>
         </is>
       </c>
       <c r="B238" s="4" t="inlineStr"/>
@@ -5783,7 +5777,7 @@
     <row r="239">
       <c r="A239" s="4" t="inlineStr">
         <is>
-          <t>01월 26일</t>
+          <t>01월 13일</t>
         </is>
       </c>
       <c r="B239" s="4" t="inlineStr"/>
@@ -5792,11 +5786,11 @@
       <c r="E239" s="4" t="inlineStr"/>
       <c r="F239" s="4" t="inlineStr"/>
       <c r="G239" s="4" t="inlineStr"/>
-      <c r="H239" s="4" t="inlineStr"/>
+      <c r="H239" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I239" s="4" t="inlineStr"/>
-      <c r="J239" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J239" s="4" t="inlineStr"/>
       <c r="K239" s="4" t="inlineStr"/>
       <c r="L239" s="5" t="n">
         <v>1</v>
@@ -5805,7 +5799,7 @@
     <row r="240">
       <c r="A240" s="4" t="inlineStr">
         <is>
-          <t>01월 25일</t>
+          <t>01월 08일</t>
         </is>
       </c>
       <c r="B240" s="4" t="inlineStr"/>
@@ -5814,10 +5808,10 @@
       <c r="E240" s="4" t="inlineStr"/>
       <c r="F240" s="4" t="inlineStr"/>
       <c r="G240" s="4" t="inlineStr"/>
-      <c r="H240" s="4" t="inlineStr"/>
-      <c r="I240" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H240" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I240" s="4" t="inlineStr"/>
       <c r="J240" s="4" t="inlineStr"/>
       <c r="K240" s="4" t="inlineStr"/>
       <c r="L240" s="5" t="n">
@@ -5827,7 +5821,7 @@
     <row r="241">
       <c r="A241" s="4" t="inlineStr">
         <is>
-          <t>01월 15일</t>
+          <t>12월 18일</t>
         </is>
       </c>
       <c r="B241" s="4" t="inlineStr"/>
@@ -5836,11 +5830,11 @@
       <c r="E241" s="4" t="inlineStr"/>
       <c r="F241" s="4" t="inlineStr"/>
       <c r="G241" s="4" t="inlineStr"/>
-      <c r="H241" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H241" s="4" t="inlineStr"/>
       <c r="I241" s="4" t="inlineStr"/>
-      <c r="J241" s="4" t="inlineStr"/>
+      <c r="J241" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K241" s="4" t="inlineStr"/>
       <c r="L241" s="5" t="n">
         <v>1</v>
@@ -5849,7 +5843,7 @@
     <row r="242">
       <c r="A242" s="4" t="inlineStr">
         <is>
-          <t>01월 13일</t>
+          <t>12월 15일</t>
         </is>
       </c>
       <c r="B242" s="4" t="inlineStr"/>
@@ -5871,7 +5865,7 @@
     <row r="243">
       <c r="A243" s="4" t="inlineStr">
         <is>
-          <t>01월 08일</t>
+          <t>12월 14일</t>
         </is>
       </c>
       <c r="B243" s="4" t="inlineStr"/>
@@ -5893,7 +5887,7 @@
     <row r="244">
       <c r="A244" s="4" t="inlineStr">
         <is>
-          <t>12월 30일</t>
+          <t>12월 11일</t>
         </is>
       </c>
       <c r="B244" s="4" t="inlineStr"/>
@@ -5902,10 +5896,10 @@
       <c r="E244" s="4" t="inlineStr"/>
       <c r="F244" s="4" t="inlineStr"/>
       <c r="G244" s="4" t="inlineStr"/>
-      <c r="H244" s="4" t="inlineStr"/>
-      <c r="I244" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H244" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I244" s="4" t="inlineStr"/>
       <c r="J244" s="4" t="inlineStr"/>
       <c r="K244" s="4" t="inlineStr"/>
       <c r="L244" s="5" t="n">
@@ -5915,7 +5909,7 @@
     <row r="245">
       <c r="A245" s="4" t="inlineStr">
         <is>
-          <t>12월 18일</t>
+          <t>12월 03일</t>
         </is>
       </c>
       <c r="B245" s="4" t="inlineStr"/>
@@ -5924,11 +5918,11 @@
       <c r="E245" s="4" t="inlineStr"/>
       <c r="F245" s="4" t="inlineStr"/>
       <c r="G245" s="4" t="inlineStr"/>
-      <c r="H245" s="4" t="inlineStr"/>
+      <c r="H245" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I245" s="4" t="inlineStr"/>
-      <c r="J245" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J245" s="4" t="inlineStr"/>
       <c r="K245" s="4" t="inlineStr"/>
       <c r="L245" s="5" t="n">
         <v>1</v>
@@ -5937,7 +5931,7 @@
     <row r="246">
       <c r="A246" s="4" t="inlineStr">
         <is>
-          <t>12월 17일</t>
+          <t>10월 15일</t>
         </is>
       </c>
       <c r="B246" s="4" t="inlineStr"/>
@@ -5946,10 +5940,10 @@
       <c r="E246" s="4" t="inlineStr"/>
       <c r="F246" s="4" t="inlineStr"/>
       <c r="G246" s="4" t="inlineStr"/>
-      <c r="H246" s="4" t="inlineStr"/>
-      <c r="I246" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H246" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I246" s="4" t="inlineStr"/>
       <c r="J246" s="4" t="inlineStr"/>
       <c r="K246" s="4" t="inlineStr"/>
       <c r="L246" s="5" t="n">
@@ -5959,7 +5953,7 @@
     <row r="247">
       <c r="A247" s="4" t="inlineStr">
         <is>
-          <t>12월 15일</t>
+          <t>09월 28일</t>
         </is>
       </c>
       <c r="B247" s="4" t="inlineStr"/>
@@ -5981,7 +5975,7 @@
     <row r="248">
       <c r="A248" s="4" t="inlineStr">
         <is>
-          <t>12월 14일</t>
+          <t>06월 04일</t>
         </is>
       </c>
       <c r="B248" s="4" t="inlineStr"/>
@@ -5993,19 +5987,17 @@
       <c r="H248" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I248" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I248" s="4" t="inlineStr"/>
       <c r="J248" s="4" t="inlineStr"/>
       <c r="K248" s="4" t="inlineStr"/>
       <c r="L248" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="4" t="inlineStr">
         <is>
-          <t>12월 11일</t>
+          <t>05월 27일</t>
         </is>
       </c>
       <c r="B249" s="4" t="inlineStr"/>
@@ -6027,7 +6019,7 @@
     <row r="250">
       <c r="A250" s="4" t="inlineStr">
         <is>
-          <t>12월 03일</t>
+          <t>05월 07일</t>
         </is>
       </c>
       <c r="B250" s="4" t="inlineStr"/>
@@ -6049,7 +6041,7 @@
     <row r="251">
       <c r="A251" s="4" t="inlineStr">
         <is>
-          <t>11월 13일</t>
+          <t>02월 27일</t>
         </is>
       </c>
       <c r="B251" s="4" t="inlineStr"/>
@@ -6058,20 +6050,20 @@
       <c r="E251" s="4" t="inlineStr"/>
       <c r="F251" s="4" t="inlineStr"/>
       <c r="G251" s="4" t="inlineStr"/>
-      <c r="H251" s="4" t="inlineStr"/>
-      <c r="I251" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H251" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I251" s="4" t="inlineStr"/>
       <c r="J251" s="4" t="inlineStr"/>
       <c r="K251" s="4" t="inlineStr"/>
       <c r="L251" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="4" t="inlineStr">
         <is>
-          <t>10월 15일</t>
+          <t>01월 20일</t>
         </is>
       </c>
       <c r="B252" s="4" t="inlineStr"/>
@@ -6093,7 +6085,7 @@
     <row r="253">
       <c r="A253" s="4" t="inlineStr">
         <is>
-          <t>09월 28일</t>
+          <t>01월 18일</t>
         </is>
       </c>
       <c r="B253" s="4" t="inlineStr"/>
@@ -6115,7 +6107,7 @@
     <row r="254">
       <c r="A254" s="4" t="inlineStr">
         <is>
-          <t>09월 25일</t>
+          <t>01월 17일</t>
         </is>
       </c>
       <c r="B254" s="4" t="inlineStr"/>
@@ -6124,10 +6116,10 @@
       <c r="E254" s="4" t="inlineStr"/>
       <c r="F254" s="4" t="inlineStr"/>
       <c r="G254" s="4" t="inlineStr"/>
-      <c r="H254" s="4" t="inlineStr"/>
-      <c r="I254" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H254" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I254" s="4" t="inlineStr"/>
       <c r="J254" s="4" t="inlineStr"/>
       <c r="K254" s="4" t="inlineStr"/>
       <c r="L254" s="5" t="n">
@@ -6137,7 +6129,7 @@
     <row r="255">
       <c r="A255" s="4" t="inlineStr">
         <is>
-          <t>07월 04일</t>
+          <t>12월 16일</t>
         </is>
       </c>
       <c r="B255" s="4" t="inlineStr"/>
@@ -6146,10 +6138,10 @@
       <c r="E255" s="4" t="inlineStr"/>
       <c r="F255" s="4" t="inlineStr"/>
       <c r="G255" s="4" t="inlineStr"/>
-      <c r="H255" s="4" t="inlineStr"/>
-      <c r="I255" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H255" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I255" s="4" t="inlineStr"/>
       <c r="J255" s="4" t="inlineStr"/>
       <c r="K255" s="4" t="inlineStr"/>
       <c r="L255" s="5" t="n">
@@ -6159,7 +6151,7 @@
     <row r="256">
       <c r="A256" s="4" t="inlineStr">
         <is>
-          <t>06월 14일</t>
+          <t>12월 06일</t>
         </is>
       </c>
       <c r="B256" s="4" t="inlineStr"/>
@@ -6168,20 +6160,20 @@
       <c r="E256" s="4" t="inlineStr"/>
       <c r="F256" s="4" t="inlineStr"/>
       <c r="G256" s="4" t="inlineStr"/>
-      <c r="H256" s="4" t="inlineStr"/>
-      <c r="I256" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H256" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I256" s="4" t="inlineStr"/>
       <c r="J256" s="4" t="inlineStr"/>
       <c r="K256" s="4" t="inlineStr"/>
       <c r="L256" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="4" t="inlineStr">
         <is>
-          <t>06월 04일</t>
+          <t>12월 05일</t>
         </is>
       </c>
       <c r="B257" s="4" t="inlineStr"/>
@@ -6191,19 +6183,19 @@
       <c r="F257" s="4" t="inlineStr"/>
       <c r="G257" s="4" t="inlineStr"/>
       <c r="H257" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I257" s="4" t="inlineStr"/>
       <c r="J257" s="4" t="inlineStr"/>
       <c r="K257" s="4" t="inlineStr"/>
       <c r="L257" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="4" t="inlineStr">
         <is>
-          <t>05월 27일</t>
+          <t>10월 26일</t>
         </is>
       </c>
       <c r="B258" s="4" t="inlineStr"/>
@@ -6225,7 +6217,7 @@
     <row r="259">
       <c r="A259" s="4" t="inlineStr">
         <is>
-          <t>05월 09일</t>
+          <t>10월 06일</t>
         </is>
       </c>
       <c r="B259" s="4" t="inlineStr"/>
@@ -6234,10 +6226,10 @@
       <c r="E259" s="4" t="inlineStr"/>
       <c r="F259" s="4" t="inlineStr"/>
       <c r="G259" s="4" t="inlineStr"/>
-      <c r="H259" s="4" t="inlineStr"/>
-      <c r="I259" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H259" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I259" s="4" t="inlineStr"/>
       <c r="J259" s="4" t="inlineStr"/>
       <c r="K259" s="4" t="inlineStr"/>
       <c r="L259" s="5" t="n">
@@ -6247,7 +6239,7 @@
     <row r="260">
       <c r="A260" s="4" t="inlineStr">
         <is>
-          <t>05월 07일</t>
+          <t>10월 04일</t>
         </is>
       </c>
       <c r="B260" s="4" t="inlineStr"/>
@@ -6269,7 +6261,7 @@
     <row r="261">
       <c r="A261" s="4" t="inlineStr">
         <is>
-          <t>02월 27일</t>
+          <t>09월 25일</t>
         </is>
       </c>
       <c r="B261" s="4" t="inlineStr"/>
@@ -6279,19 +6271,19 @@
       <c r="F261" s="4" t="inlineStr"/>
       <c r="G261" s="4" t="inlineStr"/>
       <c r="H261" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I261" s="4" t="inlineStr"/>
       <c r="J261" s="4" t="inlineStr"/>
       <c r="K261" s="4" t="inlineStr"/>
       <c r="L261" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="4" t="inlineStr">
         <is>
-          <t>01월 20일</t>
+          <t>09월 10일</t>
         </is>
       </c>
       <c r="B262" s="4" t="inlineStr"/>
@@ -6313,7 +6305,7 @@
     <row r="263">
       <c r="A263" s="4" t="inlineStr">
         <is>
-          <t>01월 18일</t>
+          <t>09월 05일</t>
         </is>
       </c>
       <c r="B263" s="4" t="inlineStr"/>
@@ -6335,7 +6327,7 @@
     <row r="264">
       <c r="A264" s="4" t="inlineStr">
         <is>
-          <t>01월 17일</t>
+          <t>08월 25일</t>
         </is>
       </c>
       <c r="B264" s="4" t="inlineStr"/>
@@ -6357,7 +6349,7 @@
     <row r="265">
       <c r="A265" s="4" t="inlineStr">
         <is>
-          <t>12월 29일</t>
+          <t>08월 24일</t>
         </is>
       </c>
       <c r="B265" s="4" t="inlineStr"/>
@@ -6366,10 +6358,10 @@
       <c r="E265" s="4" t="inlineStr"/>
       <c r="F265" s="4" t="inlineStr"/>
       <c r="G265" s="4" t="inlineStr"/>
-      <c r="H265" s="4" t="inlineStr"/>
-      <c r="I265" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H265" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I265" s="4" t="inlineStr"/>
       <c r="J265" s="4" t="inlineStr"/>
       <c r="K265" s="4" t="inlineStr"/>
       <c r="L265" s="5" t="n">
@@ -6379,7 +6371,7 @@
     <row r="266">
       <c r="A266" s="4" t="inlineStr">
         <is>
-          <t>12월 16일</t>
+          <t>08월 21일</t>
         </is>
       </c>
       <c r="B266" s="4" t="inlineStr"/>
@@ -6401,7 +6393,7 @@
     <row r="267">
       <c r="A267" s="4" t="inlineStr">
         <is>
-          <t>12월 06일</t>
+          <t>08월 12일</t>
         </is>
       </c>
       <c r="B267" s="4" t="inlineStr"/>
@@ -6411,19 +6403,19 @@
       <c r="F267" s="4" t="inlineStr"/>
       <c r="G267" s="4" t="inlineStr"/>
       <c r="H267" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I267" s="4" t="inlineStr"/>
       <c r="J267" s="4" t="inlineStr"/>
       <c r="K267" s="4" t="inlineStr"/>
       <c r="L267" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="4" t="inlineStr">
         <is>
-          <t>12월 05일</t>
+          <t>08월 11일</t>
         </is>
       </c>
       <c r="B268" s="4" t="inlineStr"/>
@@ -6433,19 +6425,19 @@
       <c r="F268" s="4" t="inlineStr"/>
       <c r="G268" s="4" t="inlineStr"/>
       <c r="H268" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I268" s="4" t="inlineStr"/>
       <c r="J268" s="4" t="inlineStr"/>
       <c r="K268" s="4" t="inlineStr"/>
       <c r="L268" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="4" t="inlineStr">
         <is>
-          <t>11월 07일</t>
+          <t>08월 09일</t>
         </is>
       </c>
       <c r="B269" s="4" t="inlineStr"/>
@@ -6454,10 +6446,10 @@
       <c r="E269" s="4" t="inlineStr"/>
       <c r="F269" s="4" t="inlineStr"/>
       <c r="G269" s="4" t="inlineStr"/>
-      <c r="H269" s="4" t="inlineStr"/>
-      <c r="I269" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H269" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I269" s="4" t="inlineStr"/>
       <c r="J269" s="4" t="inlineStr"/>
       <c r="K269" s="4" t="inlineStr"/>
       <c r="L269" s="5" t="n">
@@ -6467,7 +6459,7 @@
     <row r="270">
       <c r="A270" s="4" t="inlineStr">
         <is>
-          <t>10월 26일</t>
+          <t>08월 08일</t>
         </is>
       </c>
       <c r="B270" s="4" t="inlineStr"/>
@@ -6489,7 +6481,7 @@
     <row r="271">
       <c r="A271" s="4" t="inlineStr">
         <is>
-          <t>10월 06일</t>
+          <t>08월 02일</t>
         </is>
       </c>
       <c r="B271" s="4" t="inlineStr"/>
@@ -6498,11 +6490,11 @@
       <c r="E271" s="4" t="inlineStr"/>
       <c r="F271" s="4" t="inlineStr"/>
       <c r="G271" s="4" t="inlineStr"/>
-      <c r="H271" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H271" s="4" t="inlineStr"/>
       <c r="I271" s="4" t="inlineStr"/>
-      <c r="J271" s="4" t="inlineStr"/>
+      <c r="J271" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K271" s="4" t="inlineStr"/>
       <c r="L271" s="5" t="n">
         <v>1</v>
@@ -6511,7 +6503,7 @@
     <row r="272">
       <c r="A272" s="4" t="inlineStr">
         <is>
-          <t>10월 04일</t>
+          <t>07월 31일</t>
         </is>
       </c>
       <c r="B272" s="4" t="inlineStr"/>
@@ -6533,7 +6525,7 @@
     <row r="273">
       <c r="A273" s="4" t="inlineStr">
         <is>
-          <t>09월 25일</t>
+          <t>07월 28일</t>
         </is>
       </c>
       <c r="B273" s="4" t="inlineStr"/>
@@ -6555,7 +6547,7 @@
     <row r="274">
       <c r="A274" s="4" t="inlineStr">
         <is>
-          <t>09월 10일</t>
+          <t>07월 19일</t>
         </is>
       </c>
       <c r="B274" s="4" t="inlineStr"/>
@@ -6577,7 +6569,7 @@
     <row r="275">
       <c r="A275" s="4" t="inlineStr">
         <is>
-          <t>09월 05일</t>
+          <t>07월 17일</t>
         </is>
       </c>
       <c r="B275" s="4" t="inlineStr"/>
@@ -6599,7 +6591,7 @@
     <row r="276">
       <c r="A276" s="4" t="inlineStr">
         <is>
-          <t>09월 02일</t>
+          <t>07월 15일</t>
         </is>
       </c>
       <c r="B276" s="4" t="inlineStr"/>
@@ -6608,10 +6600,10 @@
       <c r="E276" s="4" t="inlineStr"/>
       <c r="F276" s="4" t="inlineStr"/>
       <c r="G276" s="4" t="inlineStr"/>
-      <c r="H276" s="4" t="inlineStr"/>
-      <c r="I276" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H276" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I276" s="4" t="inlineStr"/>
       <c r="J276" s="4" t="inlineStr"/>
       <c r="K276" s="4" t="inlineStr"/>
       <c r="L276" s="5" t="n">
@@ -6621,7 +6613,7 @@
     <row r="277">
       <c r="A277" s="4" t="inlineStr">
         <is>
-          <t>08월 25일</t>
+          <t>07월 12일</t>
         </is>
       </c>
       <c r="B277" s="4" t="inlineStr"/>
@@ -6643,7 +6635,7 @@
     <row r="278">
       <c r="A278" s="4" t="inlineStr">
         <is>
-          <t>08월 24일</t>
+          <t>07월 11일</t>
         </is>
       </c>
       <c r="B278" s="4" t="inlineStr"/>
@@ -6665,7 +6657,7 @@
     <row r="279">
       <c r="A279" s="4" t="inlineStr">
         <is>
-          <t>08월 21일</t>
+          <t>07월 06일</t>
         </is>
       </c>
       <c r="B279" s="4" t="inlineStr"/>
@@ -6687,7 +6679,7 @@
     <row r="280">
       <c r="A280" s="4" t="inlineStr">
         <is>
-          <t>08월 16일</t>
+          <t>07월 02일</t>
         </is>
       </c>
       <c r="B280" s="4" t="inlineStr"/>
@@ -6696,10 +6688,10 @@
       <c r="E280" s="4" t="inlineStr"/>
       <c r="F280" s="4" t="inlineStr"/>
       <c r="G280" s="4" t="inlineStr"/>
-      <c r="H280" s="4" t="inlineStr"/>
-      <c r="I280" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H280" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I280" s="4" t="inlineStr"/>
       <c r="J280" s="4" t="inlineStr"/>
       <c r="K280" s="4" t="inlineStr"/>
       <c r="L280" s="5" t="n">
@@ -6709,7 +6701,7 @@
     <row r="281">
       <c r="A281" s="4" t="inlineStr">
         <is>
-          <t>08월 12일</t>
+          <t>06월 16일</t>
         </is>
       </c>
       <c r="B281" s="4" t="inlineStr"/>
@@ -6719,21 +6711,19 @@
       <c r="F281" s="4" t="inlineStr"/>
       <c r="G281" s="4" t="inlineStr"/>
       <c r="H281" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I281" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="I281" s="4" t="inlineStr"/>
       <c r="J281" s="4" t="inlineStr"/>
       <c r="K281" s="4" t="inlineStr"/>
       <c r="L281" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="4" t="inlineStr">
         <is>
-          <t>08월 11일</t>
+          <t>06월 06일</t>
         </is>
       </c>
       <c r="B282" s="4" t="inlineStr"/>
@@ -6755,7 +6745,7 @@
     <row r="283">
       <c r="A283" s="4" t="inlineStr">
         <is>
-          <t>08월 09일</t>
+          <t>05월 30일</t>
         </is>
       </c>
       <c r="B283" s="4" t="inlineStr"/>
@@ -6764,11 +6754,11 @@
       <c r="E283" s="4" t="inlineStr"/>
       <c r="F283" s="4" t="inlineStr"/>
       <c r="G283" s="4" t="inlineStr"/>
-      <c r="H283" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H283" s="4" t="inlineStr"/>
       <c r="I283" s="4" t="inlineStr"/>
-      <c r="J283" s="4" t="inlineStr"/>
+      <c r="J283" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K283" s="4" t="inlineStr"/>
       <c r="L283" s="5" t="n">
         <v>1</v>
@@ -6777,7 +6767,7 @@
     <row r="284">
       <c r="A284" s="4" t="inlineStr">
         <is>
-          <t>08월 08일</t>
+          <t>05월 15일</t>
         </is>
       </c>
       <c r="B284" s="4" t="inlineStr"/>
@@ -6799,7 +6789,7 @@
     <row r="285">
       <c r="A285" s="4" t="inlineStr">
         <is>
-          <t>08월 02일</t>
+          <t>05월 11일</t>
         </is>
       </c>
       <c r="B285" s="4" t="inlineStr"/>
@@ -6808,11 +6798,11 @@
       <c r="E285" s="4" t="inlineStr"/>
       <c r="F285" s="4" t="inlineStr"/>
       <c r="G285" s="4" t="inlineStr"/>
-      <c r="H285" s="4" t="inlineStr"/>
+      <c r="H285" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I285" s="4" t="inlineStr"/>
-      <c r="J285" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J285" s="4" t="inlineStr"/>
       <c r="K285" s="4" t="inlineStr"/>
       <c r="L285" s="5" t="n">
         <v>1</v>
@@ -6821,7 +6811,7 @@
     <row r="286">
       <c r="A286" s="4" t="inlineStr">
         <is>
-          <t>07월 31일</t>
+          <t>04월 19일</t>
         </is>
       </c>
       <c r="B286" s="4" t="inlineStr"/>
@@ -6843,7 +6833,7 @@
     <row r="287">
       <c r="A287" s="4" t="inlineStr">
         <is>
-          <t>07월 28일</t>
+          <t>03월 24일</t>
         </is>
       </c>
       <c r="B287" s="4" t="inlineStr"/>
@@ -6865,7 +6855,7 @@
     <row r="288">
       <c r="A288" s="4" t="inlineStr">
         <is>
-          <t>07월 19일</t>
+          <t>03월 23일</t>
         </is>
       </c>
       <c r="B288" s="4" t="inlineStr"/>
@@ -6887,7 +6877,7 @@
     <row r="289">
       <c r="A289" s="4" t="inlineStr">
         <is>
-          <t>07월 17일</t>
+          <t>12월 01일</t>
         </is>
       </c>
       <c r="B289" s="4" t="inlineStr"/>
@@ -6909,7 +6899,7 @@
     <row r="290">
       <c r="A290" s="4" t="inlineStr">
         <is>
-          <t>07월 15일</t>
+          <t>11월 06일</t>
         </is>
       </c>
       <c r="B290" s="4" t="inlineStr"/>
@@ -6931,7 +6921,7 @@
     <row r="291">
       <c r="A291" s="4" t="inlineStr">
         <is>
-          <t>07월 14일</t>
+          <t>10월 27일</t>
         </is>
       </c>
       <c r="B291" s="4" t="inlineStr"/>
@@ -6940,10 +6930,10 @@
       <c r="E291" s="4" t="inlineStr"/>
       <c r="F291" s="4" t="inlineStr"/>
       <c r="G291" s="4" t="inlineStr"/>
-      <c r="H291" s="4" t="inlineStr"/>
-      <c r="I291" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H291" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I291" s="4" t="inlineStr"/>
       <c r="J291" s="4" t="inlineStr"/>
       <c r="K291" s="4" t="inlineStr"/>
       <c r="L291" s="5" t="n">
@@ -6953,7 +6943,7 @@
     <row r="292">
       <c r="A292" s="4" t="inlineStr">
         <is>
-          <t>07월 13일</t>
+          <t>08월 23일</t>
         </is>
       </c>
       <c r="B292" s="4" t="inlineStr"/>
@@ -6962,10 +6952,10 @@
       <c r="E292" s="4" t="inlineStr"/>
       <c r="F292" s="4" t="inlineStr"/>
       <c r="G292" s="4" t="inlineStr"/>
-      <c r="H292" s="4" t="inlineStr"/>
-      <c r="I292" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H292" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I292" s="4" t="inlineStr"/>
       <c r="J292" s="4" t="inlineStr"/>
       <c r="K292" s="4" t="inlineStr"/>
       <c r="L292" s="5" t="n">
@@ -6975,7 +6965,7 @@
     <row r="293">
       <c r="A293" s="4" t="inlineStr">
         <is>
-          <t>07월 12일</t>
+          <t>07월 31일</t>
         </is>
       </c>
       <c r="B293" s="4" t="inlineStr"/>
@@ -6987,19 +6977,17 @@
       <c r="H293" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I293" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I293" s="4" t="inlineStr"/>
       <c r="J293" s="4" t="inlineStr"/>
       <c r="K293" s="4" t="inlineStr"/>
       <c r="L293" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="4" t="inlineStr">
         <is>
-          <t>07월 11일</t>
+          <t>05월 16일</t>
         </is>
       </c>
       <c r="B294" s="4" t="inlineStr"/>
@@ -7011,19 +6999,17 @@
       <c r="H294" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I294" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I294" s="4" t="inlineStr"/>
       <c r="J294" s="4" t="inlineStr"/>
       <c r="K294" s="4" t="inlineStr"/>
       <c r="L294" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="4" t="inlineStr">
         <is>
-          <t>07월 07일</t>
+          <t>05월 02일</t>
         </is>
       </c>
       <c r="B295" s="4" t="inlineStr"/>
@@ -7032,20 +7018,20 @@
       <c r="E295" s="4" t="inlineStr"/>
       <c r="F295" s="4" t="inlineStr"/>
       <c r="G295" s="4" t="inlineStr"/>
-      <c r="H295" s="4" t="inlineStr"/>
-      <c r="I295" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H295" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I295" s="4" t="inlineStr"/>
       <c r="J295" s="4" t="inlineStr"/>
       <c r="K295" s="4" t="inlineStr"/>
       <c r="L295" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="4" t="inlineStr">
         <is>
-          <t>07월 06일</t>
+          <t>03월 26일</t>
         </is>
       </c>
       <c r="B296" s="4" t="inlineStr"/>
@@ -7067,7 +7053,7 @@
     <row r="297">
       <c r="A297" s="4" t="inlineStr">
         <is>
-          <t>07월 02일</t>
+          <t>02월 27일</t>
         </is>
       </c>
       <c r="B297" s="4" t="inlineStr"/>
@@ -7089,7 +7075,7 @@
     <row r="298">
       <c r="A298" s="4" t="inlineStr">
         <is>
-          <t>06월 24일</t>
+          <t>01월 29일</t>
         </is>
       </c>
       <c r="B298" s="4" t="inlineStr"/>
@@ -7098,10 +7084,10 @@
       <c r="E298" s="4" t="inlineStr"/>
       <c r="F298" s="4" t="inlineStr"/>
       <c r="G298" s="4" t="inlineStr"/>
-      <c r="H298" s="4" t="inlineStr"/>
-      <c r="I298" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H298" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I298" s="4" t="inlineStr"/>
       <c r="J298" s="4" t="inlineStr"/>
       <c r="K298" s="4" t="inlineStr"/>
       <c r="L298" s="5" t="n">
@@ -7111,7 +7097,7 @@
     <row r="299">
       <c r="A299" s="4" t="inlineStr">
         <is>
-          <t>06월 16일</t>
+          <t>01월 08일</t>
         </is>
       </c>
       <c r="B299" s="4" t="inlineStr"/>
@@ -7133,7 +7119,7 @@
     <row r="300">
       <c r="A300" s="4" t="inlineStr">
         <is>
-          <t>06월 10일</t>
+          <t>01월 04일</t>
         </is>
       </c>
       <c r="B300" s="4" t="inlineStr"/>
@@ -7142,10 +7128,10 @@
       <c r="E300" s="4" t="inlineStr"/>
       <c r="F300" s="4" t="inlineStr"/>
       <c r="G300" s="4" t="inlineStr"/>
-      <c r="H300" s="4" t="inlineStr"/>
-      <c r="I300" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H300" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I300" s="4" t="inlineStr"/>
       <c r="J300" s="4" t="inlineStr"/>
       <c r="K300" s="4" t="inlineStr"/>
       <c r="L300" s="5" t="n">
@@ -7155,7 +7141,7 @@
     <row r="301">
       <c r="A301" s="4" t="inlineStr">
         <is>
-          <t>06월 06일</t>
+          <t>01월 02일</t>
         </is>
       </c>
       <c r="B301" s="4" t="inlineStr"/>
@@ -7177,7 +7163,7 @@
     <row r="302">
       <c r="A302" s="4" t="inlineStr">
         <is>
-          <t>05월 30일</t>
+          <t>12월 28일</t>
         </is>
       </c>
       <c r="B302" s="4" t="inlineStr"/>
@@ -7186,11 +7172,11 @@
       <c r="E302" s="4" t="inlineStr"/>
       <c r="F302" s="4" t="inlineStr"/>
       <c r="G302" s="4" t="inlineStr"/>
-      <c r="H302" s="4" t="inlineStr"/>
+      <c r="H302" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I302" s="4" t="inlineStr"/>
-      <c r="J302" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="J302" s="4" t="inlineStr"/>
       <c r="K302" s="4" t="inlineStr"/>
       <c r="L302" s="5" t="n">
         <v>1</v>
@@ -7199,7 +7185,7 @@
     <row r="303">
       <c r="A303" s="4" t="inlineStr">
         <is>
-          <t>05월 15일</t>
+          <t>12월 18일</t>
         </is>
       </c>
       <c r="B303" s="4" t="inlineStr"/>
@@ -7221,7 +7207,7 @@
     <row r="304">
       <c r="A304" s="4" t="inlineStr">
         <is>
-          <t>05월 11일</t>
+          <t>10월 18일</t>
         </is>
       </c>
       <c r="B304" s="4" t="inlineStr"/>
@@ -7243,7 +7229,7 @@
     <row r="305">
       <c r="A305" s="4" t="inlineStr">
         <is>
-          <t>05월 04일</t>
+          <t>10월 08일</t>
         </is>
       </c>
       <c r="B305" s="4" t="inlineStr"/>
@@ -7252,10 +7238,10 @@
       <c r="E305" s="4" t="inlineStr"/>
       <c r="F305" s="4" t="inlineStr"/>
       <c r="G305" s="4" t="inlineStr"/>
-      <c r="H305" s="4" t="inlineStr"/>
-      <c r="I305" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H305" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I305" s="4" t="inlineStr"/>
       <c r="J305" s="4" t="inlineStr"/>
       <c r="K305" s="4" t="inlineStr"/>
       <c r="L305" s="5" t="n">
@@ -7265,7 +7251,7 @@
     <row r="306">
       <c r="A306" s="4" t="inlineStr">
         <is>
-          <t>04월 30일</t>
+          <t>09월 28일</t>
         </is>
       </c>
       <c r="B306" s="4" t="inlineStr"/>
@@ -7274,10 +7260,10 @@
       <c r="E306" s="4" t="inlineStr"/>
       <c r="F306" s="4" t="inlineStr"/>
       <c r="G306" s="4" t="inlineStr"/>
-      <c r="H306" s="4" t="inlineStr"/>
-      <c r="I306" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H306" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I306" s="4" t="inlineStr"/>
       <c r="J306" s="4" t="inlineStr"/>
       <c r="K306" s="4" t="inlineStr"/>
       <c r="L306" s="5" t="n">
@@ -7287,7 +7273,7 @@
     <row r="307">
       <c r="A307" s="4" t="inlineStr">
         <is>
-          <t>04월 19일</t>
+          <t>09월 07일</t>
         </is>
       </c>
       <c r="B307" s="4" t="inlineStr"/>
@@ -7309,7 +7295,7 @@
     <row r="308">
       <c r="A308" s="4" t="inlineStr">
         <is>
-          <t>03월 24일</t>
+          <t>08월 21일</t>
         </is>
       </c>
       <c r="B308" s="4" t="inlineStr"/>
@@ -7331,7 +7317,7 @@
     <row r="309">
       <c r="A309" s="4" t="inlineStr">
         <is>
-          <t>03월 23일</t>
+          <t>07월 31일</t>
         </is>
       </c>
       <c r="B309" s="4" t="inlineStr"/>
@@ -7353,7 +7339,7 @@
     <row r="310">
       <c r="A310" s="4" t="inlineStr">
         <is>
-          <t>03월 12일</t>
+          <t>07월 27일</t>
         </is>
       </c>
       <c r="B310" s="4" t="inlineStr"/>
@@ -7362,10 +7348,10 @@
       <c r="E310" s="4" t="inlineStr"/>
       <c r="F310" s="4" t="inlineStr"/>
       <c r="G310" s="4" t="inlineStr"/>
-      <c r="H310" s="4" t="inlineStr"/>
-      <c r="I310" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H310" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I310" s="4" t="inlineStr"/>
       <c r="J310" s="4" t="inlineStr"/>
       <c r="K310" s="4" t="inlineStr"/>
       <c r="L310" s="5" t="n">
@@ -7375,7 +7361,7 @@
     <row r="311">
       <c r="A311" s="4" t="inlineStr">
         <is>
-          <t>02월 27일</t>
+          <t>07월 20일</t>
         </is>
       </c>
       <c r="B311" s="4" t="inlineStr"/>
@@ -7384,10 +7370,10 @@
       <c r="E311" s="4" t="inlineStr"/>
       <c r="F311" s="4" t="inlineStr"/>
       <c r="G311" s="4" t="inlineStr"/>
-      <c r="H311" s="4" t="inlineStr"/>
-      <c r="I311" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H311" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I311" s="4" t="inlineStr"/>
       <c r="J311" s="4" t="inlineStr"/>
       <c r="K311" s="4" t="inlineStr"/>
       <c r="L311" s="5" t="n">
@@ -7397,7 +7383,7 @@
     <row r="312">
       <c r="A312" s="4" t="inlineStr">
         <is>
-          <t>02월 24일</t>
+          <t>07월 19일</t>
         </is>
       </c>
       <c r="B312" s="4" t="inlineStr"/>
@@ -7406,10 +7392,10 @@
       <c r="E312" s="4" t="inlineStr"/>
       <c r="F312" s="4" t="inlineStr"/>
       <c r="G312" s="4" t="inlineStr"/>
-      <c r="H312" s="4" t="inlineStr"/>
-      <c r="I312" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H312" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I312" s="4" t="inlineStr"/>
       <c r="J312" s="4" t="inlineStr"/>
       <c r="K312" s="4" t="inlineStr"/>
       <c r="L312" s="5" t="n">
@@ -7419,7 +7405,7 @@
     <row r="313">
       <c r="A313" s="4" t="inlineStr">
         <is>
-          <t>02월 06일</t>
+          <t>07월 10일</t>
         </is>
       </c>
       <c r="B313" s="4" t="inlineStr"/>
@@ -7428,10 +7414,10 @@
       <c r="E313" s="4" t="inlineStr"/>
       <c r="F313" s="4" t="inlineStr"/>
       <c r="G313" s="4" t="inlineStr"/>
-      <c r="H313" s="4" t="inlineStr"/>
-      <c r="I313" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H313" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I313" s="4" t="inlineStr"/>
       <c r="J313" s="4" t="inlineStr"/>
       <c r="K313" s="4" t="inlineStr"/>
       <c r="L313" s="5" t="n">
@@ -7441,7 +7427,7 @@
     <row r="314">
       <c r="A314" s="4" t="inlineStr">
         <is>
-          <t>12월 02일</t>
+          <t>07월 06일</t>
         </is>
       </c>
       <c r="B314" s="4" t="inlineStr"/>
@@ -7450,10 +7436,10 @@
       <c r="E314" s="4" t="inlineStr"/>
       <c r="F314" s="4" t="inlineStr"/>
       <c r="G314" s="4" t="inlineStr"/>
-      <c r="H314" s="4" t="inlineStr"/>
-      <c r="I314" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H314" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I314" s="4" t="inlineStr"/>
       <c r="J314" s="4" t="inlineStr"/>
       <c r="K314" s="4" t="inlineStr"/>
       <c r="L314" s="5" t="n">
@@ -7463,7 +7449,7 @@
     <row r="315">
       <c r="A315" s="4" t="inlineStr">
         <is>
-          <t>12월 01일</t>
+          <t>07월 01일</t>
         </is>
       </c>
       <c r="B315" s="4" t="inlineStr"/>
@@ -7485,7 +7471,7 @@
     <row r="316">
       <c r="A316" s="4" t="inlineStr">
         <is>
-          <t>11월 06일</t>
+          <t>06월 27일</t>
         </is>
       </c>
       <c r="B316" s="4" t="inlineStr"/>
@@ -7495,19 +7481,19 @@
       <c r="F316" s="4" t="inlineStr"/>
       <c r="G316" s="4" t="inlineStr"/>
       <c r="H316" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I316" s="4" t="inlineStr"/>
       <c r="J316" s="4" t="inlineStr"/>
       <c r="K316" s="4" t="inlineStr"/>
       <c r="L316" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="317">
       <c r="A317" s="4" t="inlineStr">
         <is>
-          <t>10월 27일</t>
+          <t>06월 26일</t>
         </is>
       </c>
       <c r="B317" s="4" t="inlineStr"/>
@@ -7529,7 +7515,7 @@
     <row r="318">
       <c r="A318" s="4" t="inlineStr">
         <is>
-          <t>10월 23일</t>
+          <t>06월 16일</t>
         </is>
       </c>
       <c r="B318" s="4" t="inlineStr"/>
@@ -7538,10 +7524,10 @@
       <c r="E318" s="4" t="inlineStr"/>
       <c r="F318" s="4" t="inlineStr"/>
       <c r="G318" s="4" t="inlineStr"/>
-      <c r="H318" s="4" t="inlineStr"/>
-      <c r="I318" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H318" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I318" s="4" t="inlineStr"/>
       <c r="J318" s="4" t="inlineStr"/>
       <c r="K318" s="4" t="inlineStr"/>
       <c r="L318" s="5" t="n">
@@ -7551,7 +7537,7 @@
     <row r="319">
       <c r="A319" s="4" t="inlineStr">
         <is>
-          <t>10월 09일</t>
+          <t>06월 13일</t>
         </is>
       </c>
       <c r="B319" s="4" t="inlineStr"/>
@@ -7560,10 +7546,10 @@
       <c r="E319" s="4" t="inlineStr"/>
       <c r="F319" s="4" t="inlineStr"/>
       <c r="G319" s="4" t="inlineStr"/>
-      <c r="H319" s="4" t="inlineStr"/>
-      <c r="I319" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H319" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I319" s="4" t="inlineStr"/>
       <c r="J319" s="4" t="inlineStr"/>
       <c r="K319" s="4" t="inlineStr"/>
       <c r="L319" s="5" t="n">
@@ -7573,7 +7559,7 @@
     <row r="320">
       <c r="A320" s="4" t="inlineStr">
         <is>
-          <t>09월 30일</t>
+          <t>05월 16일</t>
         </is>
       </c>
       <c r="B320" s="4" t="inlineStr"/>
@@ -7582,10 +7568,10 @@
       <c r="E320" s="4" t="inlineStr"/>
       <c r="F320" s="4" t="inlineStr"/>
       <c r="G320" s="4" t="inlineStr"/>
-      <c r="H320" s="4" t="inlineStr"/>
-      <c r="I320" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H320" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I320" s="4" t="inlineStr"/>
       <c r="J320" s="4" t="inlineStr"/>
       <c r="K320" s="4" t="inlineStr"/>
       <c r="L320" s="5" t="n">
@@ -7595,7 +7581,7 @@
     <row r="321">
       <c r="A321" s="4" t="inlineStr">
         <is>
-          <t>08월 23일</t>
+          <t>05월 10일</t>
         </is>
       </c>
       <c r="B321" s="4" t="inlineStr"/>
@@ -7617,7 +7603,7 @@
     <row r="322">
       <c r="A322" s="4" t="inlineStr">
         <is>
-          <t>08월 10일</t>
+          <t>05월 04일</t>
         </is>
       </c>
       <c r="B322" s="4" t="inlineStr"/>
@@ -7626,10 +7612,10 @@
       <c r="E322" s="4" t="inlineStr"/>
       <c r="F322" s="4" t="inlineStr"/>
       <c r="G322" s="4" t="inlineStr"/>
-      <c r="H322" s="4" t="inlineStr"/>
-      <c r="I322" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H322" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I322" s="4" t="inlineStr"/>
       <c r="J322" s="4" t="inlineStr"/>
       <c r="K322" s="4" t="inlineStr"/>
       <c r="L322" s="5" t="n">
@@ -7639,7 +7625,7 @@
     <row r="323">
       <c r="A323" s="4" t="inlineStr">
         <is>
-          <t>08월 01일</t>
+          <t>04월 20일</t>
         </is>
       </c>
       <c r="B323" s="4" t="inlineStr"/>
@@ -7648,10 +7634,10 @@
       <c r="E323" s="4" t="inlineStr"/>
       <c r="F323" s="4" t="inlineStr"/>
       <c r="G323" s="4" t="inlineStr"/>
-      <c r="H323" s="4" t="inlineStr"/>
-      <c r="I323" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H323" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I323" s="4" t="inlineStr"/>
       <c r="J323" s="4" t="inlineStr"/>
       <c r="K323" s="4" t="inlineStr"/>
       <c r="L323" s="5" t="n">
@@ -7661,7 +7647,7 @@
     <row r="324">
       <c r="A324" s="4" t="inlineStr">
         <is>
-          <t>07월 31일</t>
+          <t>04월 06일</t>
         </is>
       </c>
       <c r="B324" s="4" t="inlineStr"/>
@@ -7683,7 +7669,7 @@
     <row r="325">
       <c r="A325" s="4" t="inlineStr">
         <is>
-          <t>07월 27일</t>
+          <t>03월 31일</t>
         </is>
       </c>
       <c r="B325" s="4" t="inlineStr"/>
@@ -7692,10 +7678,10 @@
       <c r="E325" s="4" t="inlineStr"/>
       <c r="F325" s="4" t="inlineStr"/>
       <c r="G325" s="4" t="inlineStr"/>
-      <c r="H325" s="4" t="inlineStr"/>
-      <c r="I325" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H325" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I325" s="4" t="inlineStr"/>
       <c r="J325" s="4" t="inlineStr"/>
       <c r="K325" s="4" t="inlineStr"/>
       <c r="L325" s="5" t="n">
@@ -7705,7 +7691,7 @@
     <row r="326">
       <c r="A326" s="4" t="inlineStr">
         <is>
-          <t>07월 11일</t>
+          <t>03월 25일</t>
         </is>
       </c>
       <c r="B326" s="4" t="inlineStr"/>
@@ -7714,10 +7700,10 @@
       <c r="E326" s="4" t="inlineStr"/>
       <c r="F326" s="4" t="inlineStr"/>
       <c r="G326" s="4" t="inlineStr"/>
-      <c r="H326" s="4" t="inlineStr"/>
-      <c r="I326" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H326" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I326" s="4" t="inlineStr"/>
       <c r="J326" s="4" t="inlineStr"/>
       <c r="K326" s="4" t="inlineStr"/>
       <c r="L326" s="5" t="n">
@@ -7727,7 +7713,7 @@
     <row r="327">
       <c r="A327" s="4" t="inlineStr">
         <is>
-          <t>05월 16일</t>
+          <t>03월 21일</t>
         </is>
       </c>
       <c r="B327" s="4" t="inlineStr"/>
@@ -7749,7 +7735,7 @@
     <row r="328">
       <c r="A328" s="4" t="inlineStr">
         <is>
-          <t>05월 02일</t>
+          <t>02월 24일</t>
         </is>
       </c>
       <c r="B328" s="4" t="inlineStr"/>
@@ -7759,19 +7745,19 @@
       <c r="F328" s="4" t="inlineStr"/>
       <c r="G328" s="4" t="inlineStr"/>
       <c r="H328" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I328" s="4" t="inlineStr"/>
       <c r="J328" s="4" t="inlineStr"/>
       <c r="K328" s="4" t="inlineStr"/>
       <c r="L328" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" s="4" t="inlineStr">
         <is>
-          <t>03월 26일</t>
+          <t>01월 31일</t>
         </is>
       </c>
       <c r="B329" s="4" t="inlineStr"/>
@@ -7793,7 +7779,7 @@
     <row r="330">
       <c r="A330" s="4" t="inlineStr">
         <is>
-          <t>02월 27일</t>
+          <t>01월 24일</t>
         </is>
       </c>
       <c r="B330" s="4" t="inlineStr"/>
@@ -7815,7 +7801,7 @@
     <row r="331">
       <c r="A331" s="4" t="inlineStr">
         <is>
-          <t>01월 29일</t>
+          <t>01월 20일</t>
         </is>
       </c>
       <c r="B331" s="4" t="inlineStr"/>
@@ -7825,19 +7811,19 @@
       <c r="F331" s="4" t="inlineStr"/>
       <c r="G331" s="4" t="inlineStr"/>
       <c r="H331" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I331" s="4" t="inlineStr"/>
       <c r="J331" s="4" t="inlineStr"/>
       <c r="K331" s="4" t="inlineStr"/>
       <c r="L331" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="332">
       <c r="A332" s="4" t="inlineStr">
         <is>
-          <t>01월 08일</t>
+          <t>01월 12일</t>
         </is>
       </c>
       <c r="B332" s="4" t="inlineStr"/>
@@ -7859,7 +7845,7 @@
     <row r="333">
       <c r="A333" s="4" t="inlineStr">
         <is>
-          <t>01월 04일</t>
+          <t>01월 03일</t>
         </is>
       </c>
       <c r="B333" s="4" t="inlineStr"/>
@@ -7881,7 +7867,7 @@
     <row r="334">
       <c r="A334" s="4" t="inlineStr">
         <is>
-          <t>01월 02일</t>
+          <t>12월 19일</t>
         </is>
       </c>
       <c r="B334" s="4" t="inlineStr"/>
@@ -7903,7 +7889,7 @@
     <row r="335">
       <c r="A335" s="4" t="inlineStr">
         <is>
-          <t>12월 28일</t>
+          <t>12월 08일</t>
         </is>
       </c>
       <c r="B335" s="4" t="inlineStr"/>
@@ -7925,7 +7911,7 @@
     <row r="336">
       <c r="A336" s="4" t="inlineStr">
         <is>
-          <t>12월 18일</t>
+          <t>11월 10일</t>
         </is>
       </c>
       <c r="B336" s="4" t="inlineStr"/>
@@ -7934,11 +7920,11 @@
       <c r="E336" s="4" t="inlineStr"/>
       <c r="F336" s="4" t="inlineStr"/>
       <c r="G336" s="4" t="inlineStr"/>
-      <c r="H336" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H336" s="4" t="inlineStr"/>
       <c r="I336" s="4" t="inlineStr"/>
-      <c r="J336" s="4" t="inlineStr"/>
+      <c r="J336" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K336" s="4" t="inlineStr"/>
       <c r="L336" s="5" t="n">
         <v>1</v>
@@ -7947,7 +7933,7 @@
     <row r="337">
       <c r="A337" s="4" t="inlineStr">
         <is>
-          <t>11월 20일</t>
+          <t>11월 08일</t>
         </is>
       </c>
       <c r="B337" s="4" t="inlineStr"/>
@@ -7956,10 +7942,10 @@
       <c r="E337" s="4" t="inlineStr"/>
       <c r="F337" s="4" t="inlineStr"/>
       <c r="G337" s="4" t="inlineStr"/>
-      <c r="H337" s="4" t="inlineStr"/>
-      <c r="I337" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H337" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I337" s="4" t="inlineStr"/>
       <c r="J337" s="4" t="inlineStr"/>
       <c r="K337" s="4" t="inlineStr"/>
       <c r="L337" s="5" t="n">
@@ -7969,7 +7955,7 @@
     <row r="338">
       <c r="A338" s="4" t="inlineStr">
         <is>
-          <t>10월 18일</t>
+          <t>10월 26일</t>
         </is>
       </c>
       <c r="B338" s="4" t="inlineStr"/>
@@ -7991,7 +7977,7 @@
     <row r="339">
       <c r="A339" s="4" t="inlineStr">
         <is>
-          <t>10월 08일</t>
+          <t>10월 24일</t>
         </is>
       </c>
       <c r="B339" s="4" t="inlineStr"/>
@@ -8013,7 +7999,7 @@
     <row r="340">
       <c r="A340" s="4" t="inlineStr">
         <is>
-          <t>09월 28일</t>
+          <t>10월 18일</t>
         </is>
       </c>
       <c r="B340" s="4" t="inlineStr"/>
@@ -8023,19 +8009,19 @@
       <c r="F340" s="4" t="inlineStr"/>
       <c r="G340" s="4" t="inlineStr"/>
       <c r="H340" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I340" s="4" t="inlineStr"/>
       <c r="J340" s="4" t="inlineStr"/>
       <c r="K340" s="4" t="inlineStr"/>
       <c r="L340" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="341">
       <c r="A341" s="4" t="inlineStr">
         <is>
-          <t>09월 07일</t>
+          <t>10월 17일</t>
         </is>
       </c>
       <c r="B341" s="4" t="inlineStr"/>
@@ -8057,7 +8043,7 @@
     <row r="342">
       <c r="A342" s="4" t="inlineStr">
         <is>
-          <t>08월 21일</t>
+          <t>10월 03일</t>
         </is>
       </c>
       <c r="B342" s="4" t="inlineStr"/>
@@ -8079,7 +8065,7 @@
     <row r="343">
       <c r="A343" s="4" t="inlineStr">
         <is>
-          <t>07월 31일</t>
+          <t>09월 28일</t>
         </is>
       </c>
       <c r="B343" s="4" t="inlineStr"/>
@@ -8091,19 +8077,17 @@
       <c r="H343" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="I343" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="I343" s="4" t="inlineStr"/>
       <c r="J343" s="4" t="inlineStr"/>
       <c r="K343" s="4" t="inlineStr"/>
       <c r="L343" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" s="4" t="inlineStr">
         <is>
-          <t>07월 27일</t>
+          <t>09월 24일</t>
         </is>
       </c>
       <c r="B344" s="4" t="inlineStr"/>
@@ -8125,7 +8109,7 @@
     <row r="345">
       <c r="A345" s="4" t="inlineStr">
         <is>
-          <t>07월 20일</t>
+          <t>09월 19일</t>
         </is>
       </c>
       <c r="B345" s="4" t="inlineStr"/>
@@ -8147,7 +8131,7 @@
     <row r="346">
       <c r="A346" s="4" t="inlineStr">
         <is>
-          <t>07월 19일</t>
+          <t>09월 02일</t>
         </is>
       </c>
       <c r="B346" s="4" t="inlineStr"/>
@@ -8156,11 +8140,11 @@
       <c r="E346" s="4" t="inlineStr"/>
       <c r="F346" s="4" t="inlineStr"/>
       <c r="G346" s="4" t="inlineStr"/>
-      <c r="H346" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H346" s="4" t="inlineStr"/>
       <c r="I346" s="4" t="inlineStr"/>
-      <c r="J346" s="4" t="inlineStr"/>
+      <c r="J346" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K346" s="4" t="inlineStr"/>
       <c r="L346" s="5" t="n">
         <v>1</v>
@@ -8169,7 +8153,7 @@
     <row r="347">
       <c r="A347" s="4" t="inlineStr">
         <is>
-          <t>07월 10일</t>
+          <t>06월 16일</t>
         </is>
       </c>
       <c r="B347" s="4" t="inlineStr"/>
@@ -8178,11 +8162,11 @@
       <c r="E347" s="4" t="inlineStr"/>
       <c r="F347" s="4" t="inlineStr"/>
       <c r="G347" s="4" t="inlineStr"/>
-      <c r="H347" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H347" s="4" t="inlineStr"/>
       <c r="I347" s="4" t="inlineStr"/>
-      <c r="J347" s="4" t="inlineStr"/>
+      <c r="J347" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K347" s="4" t="inlineStr"/>
       <c r="L347" s="5" t="n">
         <v>1</v>
@@ -8191,7 +8175,7 @@
     <row r="348">
       <c r="A348" s="4" t="inlineStr">
         <is>
-          <t>07월 06일</t>
+          <t>11월 28일</t>
         </is>
       </c>
       <c r="B348" s="4" t="inlineStr"/>
@@ -8200,11 +8184,11 @@
       <c r="E348" s="4" t="inlineStr"/>
       <c r="F348" s="4" t="inlineStr"/>
       <c r="G348" s="4" t="inlineStr"/>
-      <c r="H348" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H348" s="4" t="inlineStr"/>
       <c r="I348" s="4" t="inlineStr"/>
-      <c r="J348" s="4" t="inlineStr"/>
+      <c r="J348" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K348" s="4" t="inlineStr"/>
       <c r="L348" s="5" t="n">
         <v>1</v>
@@ -8213,7 +8197,7 @@
     <row r="349">
       <c r="A349" s="4" t="inlineStr">
         <is>
-          <t>07월 01일</t>
+          <t>11월 21일</t>
         </is>
       </c>
       <c r="B349" s="4" t="inlineStr"/>
@@ -8222,11 +8206,11 @@
       <c r="E349" s="4" t="inlineStr"/>
       <c r="F349" s="4" t="inlineStr"/>
       <c r="G349" s="4" t="inlineStr"/>
-      <c r="H349" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H349" s="4" t="inlineStr"/>
       <c r="I349" s="4" t="inlineStr"/>
-      <c r="J349" s="4" t="inlineStr"/>
+      <c r="J349" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K349" s="4" t="inlineStr"/>
       <c r="L349" s="5" t="n">
         <v>1</v>
@@ -8235,7 +8219,7 @@
     <row r="350">
       <c r="A350" s="4" t="inlineStr">
         <is>
-          <t>06월 27일</t>
+          <t>11월 18일</t>
         </is>
       </c>
       <c r="B350" s="4" t="inlineStr"/>
@@ -8244,20 +8228,20 @@
       <c r="E350" s="4" t="inlineStr"/>
       <c r="F350" s="4" t="inlineStr"/>
       <c r="G350" s="4" t="inlineStr"/>
-      <c r="H350" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="H350" s="4" t="inlineStr"/>
       <c r="I350" s="4" t="inlineStr"/>
-      <c r="J350" s="4" t="inlineStr"/>
+      <c r="J350" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K350" s="4" t="inlineStr"/>
       <c r="L350" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="351">
       <c r="A351" s="4" t="inlineStr">
         <is>
-          <t>06월 26일</t>
+          <t>11월 27일</t>
         </is>
       </c>
       <c r="B351" s="4" t="inlineStr"/>
@@ -8266,11 +8250,11 @@
       <c r="E351" s="4" t="inlineStr"/>
       <c r="F351" s="4" t="inlineStr"/>
       <c r="G351" s="4" t="inlineStr"/>
-      <c r="H351" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H351" s="4" t="inlineStr"/>
       <c r="I351" s="4" t="inlineStr"/>
-      <c r="J351" s="4" t="inlineStr"/>
+      <c r="J351" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K351" s="4" t="inlineStr"/>
       <c r="L351" s="5" t="n">
         <v>1</v>
@@ -8279,7 +8263,7 @@
     <row r="352">
       <c r="A352" s="4" t="inlineStr">
         <is>
-          <t>06월 16일</t>
+          <t>02월 11일</t>
         </is>
       </c>
       <c r="B352" s="4" t="inlineStr"/>
@@ -8288,794 +8272,44 @@
       <c r="E352" s="4" t="inlineStr"/>
       <c r="F352" s="4" t="inlineStr"/>
       <c r="G352" s="4" t="inlineStr"/>
-      <c r="H352" s="4" t="n">
-        <v>1</v>
-      </c>
+      <c r="H352" s="4" t="inlineStr"/>
       <c r="I352" s="4" t="inlineStr"/>
-      <c r="J352" s="4" t="inlineStr"/>
+      <c r="J352" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="K352" s="4" t="inlineStr"/>
       <c r="L352" s="5" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="353">
-      <c r="A353" s="4" t="inlineStr">
-        <is>
-          <t>06월 13일</t>
-        </is>
-      </c>
-      <c r="B353" s="4" t="inlineStr"/>
-      <c r="C353" s="4" t="inlineStr"/>
-      <c r="D353" s="4" t="inlineStr"/>
-      <c r="E353" s="4" t="inlineStr"/>
-      <c r="F353" s="4" t="inlineStr"/>
-      <c r="G353" s="4" t="inlineStr"/>
-      <c r="H353" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I353" s="4" t="inlineStr"/>
-      <c r="J353" s="4" t="inlineStr"/>
-      <c r="K353" s="4" t="inlineStr"/>
-      <c r="L353" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" s="4" t="inlineStr">
-        <is>
-          <t>05월 16일</t>
-        </is>
-      </c>
-      <c r="B354" s="4" t="inlineStr"/>
-      <c r="C354" s="4" t="inlineStr"/>
-      <c r="D354" s="4" t="inlineStr"/>
-      <c r="E354" s="4" t="inlineStr"/>
-      <c r="F354" s="4" t="inlineStr"/>
-      <c r="G354" s="4" t="inlineStr"/>
-      <c r="H354" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I354" s="4" t="inlineStr"/>
-      <c r="J354" s="4" t="inlineStr"/>
-      <c r="K354" s="4" t="inlineStr"/>
-      <c r="L354" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="355">
-      <c r="A355" s="4" t="inlineStr">
-        <is>
-          <t>05월 10일</t>
-        </is>
-      </c>
-      <c r="B355" s="4" t="inlineStr"/>
-      <c r="C355" s="4" t="inlineStr"/>
-      <c r="D355" s="4" t="inlineStr"/>
-      <c r="E355" s="4" t="inlineStr"/>
-      <c r="F355" s="4" t="inlineStr"/>
-      <c r="G355" s="4" t="inlineStr"/>
-      <c r="H355" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I355" s="4" t="inlineStr"/>
-      <c r="J355" s="4" t="inlineStr"/>
-      <c r="K355" s="4" t="inlineStr"/>
-      <c r="L355" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" s="4" t="inlineStr">
-        <is>
-          <t>05월 04일</t>
-        </is>
-      </c>
-      <c r="B356" s="4" t="inlineStr"/>
-      <c r="C356" s="4" t="inlineStr"/>
-      <c r="D356" s="4" t="inlineStr"/>
-      <c r="E356" s="4" t="inlineStr"/>
-      <c r="F356" s="4" t="inlineStr"/>
-      <c r="G356" s="4" t="inlineStr"/>
-      <c r="H356" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I356" s="4" t="inlineStr"/>
-      <c r="J356" s="4" t="inlineStr"/>
-      <c r="K356" s="4" t="inlineStr"/>
-      <c r="L356" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" s="4" t="inlineStr">
-        <is>
-          <t>04월 20일</t>
-        </is>
-      </c>
-      <c r="B357" s="4" t="inlineStr"/>
-      <c r="C357" s="4" t="inlineStr"/>
-      <c r="D357" s="4" t="inlineStr"/>
-      <c r="E357" s="4" t="inlineStr"/>
-      <c r="F357" s="4" t="inlineStr"/>
-      <c r="G357" s="4" t="inlineStr"/>
-      <c r="H357" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I357" s="4" t="inlineStr"/>
-      <c r="J357" s="4" t="inlineStr"/>
-      <c r="K357" s="4" t="inlineStr"/>
-      <c r="L357" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" s="4" t="inlineStr">
-        <is>
-          <t>04월 06일</t>
-        </is>
-      </c>
-      <c r="B358" s="4" t="inlineStr"/>
-      <c r="C358" s="4" t="inlineStr"/>
-      <c r="D358" s="4" t="inlineStr"/>
-      <c r="E358" s="4" t="inlineStr"/>
-      <c r="F358" s="4" t="inlineStr"/>
-      <c r="G358" s="4" t="inlineStr"/>
-      <c r="H358" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I358" s="4" t="inlineStr"/>
-      <c r="J358" s="4" t="inlineStr"/>
-      <c r="K358" s="4" t="inlineStr"/>
-      <c r="L358" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" s="4" t="inlineStr">
-        <is>
-          <t>03월 31일</t>
-        </is>
-      </c>
-      <c r="B359" s="4" t="inlineStr"/>
-      <c r="C359" s="4" t="inlineStr"/>
-      <c r="D359" s="4" t="inlineStr"/>
-      <c r="E359" s="4" t="inlineStr"/>
-      <c r="F359" s="4" t="inlineStr"/>
-      <c r="G359" s="4" t="inlineStr"/>
-      <c r="H359" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I359" s="4" t="inlineStr"/>
-      <c r="J359" s="4" t="inlineStr"/>
-      <c r="K359" s="4" t="inlineStr"/>
-      <c r="L359" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="360">
-      <c r="A360" s="4" t="inlineStr">
-        <is>
-          <t>03월 25일</t>
-        </is>
-      </c>
-      <c r="B360" s="4" t="inlineStr"/>
-      <c r="C360" s="4" t="inlineStr"/>
-      <c r="D360" s="4" t="inlineStr"/>
-      <c r="E360" s="4" t="inlineStr"/>
-      <c r="F360" s="4" t="inlineStr"/>
-      <c r="G360" s="4" t="inlineStr"/>
-      <c r="H360" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I360" s="4" t="inlineStr"/>
-      <c r="J360" s="4" t="inlineStr"/>
-      <c r="K360" s="4" t="inlineStr"/>
-      <c r="L360" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="361">
-      <c r="A361" s="4" t="inlineStr">
-        <is>
-          <t>03월 21일</t>
-        </is>
-      </c>
-      <c r="B361" s="4" t="inlineStr"/>
-      <c r="C361" s="4" t="inlineStr"/>
-      <c r="D361" s="4" t="inlineStr"/>
-      <c r="E361" s="4" t="inlineStr"/>
-      <c r="F361" s="4" t="inlineStr"/>
-      <c r="G361" s="4" t="inlineStr"/>
-      <c r="H361" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I361" s="4" t="inlineStr"/>
-      <c r="J361" s="4" t="inlineStr"/>
-      <c r="K361" s="4" t="inlineStr"/>
-      <c r="L361" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="362">
-      <c r="A362" s="4" t="inlineStr">
-        <is>
-          <t>02월 24일</t>
-        </is>
-      </c>
-      <c r="B362" s="4" t="inlineStr"/>
-      <c r="C362" s="4" t="inlineStr"/>
-      <c r="D362" s="4" t="inlineStr"/>
-      <c r="E362" s="4" t="inlineStr"/>
-      <c r="F362" s="4" t="inlineStr"/>
-      <c r="G362" s="4" t="inlineStr"/>
-      <c r="H362" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I362" s="4" t="inlineStr"/>
-      <c r="J362" s="4" t="inlineStr"/>
-      <c r="K362" s="4" t="inlineStr"/>
-      <c r="L362" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="363">
-      <c r="A363" s="4" t="inlineStr">
-        <is>
-          <t>01월 31일</t>
-        </is>
-      </c>
-      <c r="B363" s="4" t="inlineStr"/>
-      <c r="C363" s="4" t="inlineStr"/>
-      <c r="D363" s="4" t="inlineStr"/>
-      <c r="E363" s="4" t="inlineStr"/>
-      <c r="F363" s="4" t="inlineStr"/>
-      <c r="G363" s="4" t="inlineStr"/>
-      <c r="H363" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I363" s="4" t="inlineStr"/>
-      <c r="J363" s="4" t="inlineStr"/>
-      <c r="K363" s="4" t="inlineStr"/>
-      <c r="L363" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="364">
-      <c r="A364" s="4" t="inlineStr">
-        <is>
-          <t>01월 24일</t>
-        </is>
-      </c>
-      <c r="B364" s="4" t="inlineStr"/>
-      <c r="C364" s="4" t="inlineStr"/>
-      <c r="D364" s="4" t="inlineStr"/>
-      <c r="E364" s="4" t="inlineStr"/>
-      <c r="F364" s="4" t="inlineStr"/>
-      <c r="G364" s="4" t="inlineStr"/>
-      <c r="H364" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I364" s="4" t="inlineStr"/>
-      <c r="J364" s="4" t="inlineStr"/>
-      <c r="K364" s="4" t="inlineStr"/>
-      <c r="L364" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="365">
-      <c r="A365" s="4" t="inlineStr">
-        <is>
-          <t>01월 20일</t>
-        </is>
-      </c>
-      <c r="B365" s="4" t="inlineStr"/>
-      <c r="C365" s="4" t="inlineStr"/>
-      <c r="D365" s="4" t="inlineStr"/>
-      <c r="E365" s="4" t="inlineStr"/>
-      <c r="F365" s="4" t="inlineStr"/>
-      <c r="G365" s="4" t="inlineStr"/>
-      <c r="H365" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I365" s="4" t="inlineStr"/>
-      <c r="J365" s="4" t="inlineStr"/>
-      <c r="K365" s="4" t="inlineStr"/>
-      <c r="L365" s="5" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="366">
-      <c r="A366" s="4" t="inlineStr">
-        <is>
-          <t>01월 12일</t>
-        </is>
-      </c>
-      <c r="B366" s="4" t="inlineStr"/>
-      <c r="C366" s="4" t="inlineStr"/>
-      <c r="D366" s="4" t="inlineStr"/>
-      <c r="E366" s="4" t="inlineStr"/>
-      <c r="F366" s="4" t="inlineStr"/>
-      <c r="G366" s="4" t="inlineStr"/>
-      <c r="H366" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I366" s="4" t="inlineStr"/>
-      <c r="J366" s="4" t="inlineStr"/>
-      <c r="K366" s="4" t="inlineStr"/>
-      <c r="L366" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="367">
-      <c r="A367" s="4" t="inlineStr">
-        <is>
-          <t>01월 03일</t>
-        </is>
-      </c>
-      <c r="B367" s="4" t="inlineStr"/>
-      <c r="C367" s="4" t="inlineStr"/>
-      <c r="D367" s="4" t="inlineStr"/>
-      <c r="E367" s="4" t="inlineStr"/>
-      <c r="F367" s="4" t="inlineStr"/>
-      <c r="G367" s="4" t="inlineStr"/>
-      <c r="H367" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I367" s="4" t="inlineStr"/>
-      <c r="J367" s="4" t="inlineStr"/>
-      <c r="K367" s="4" t="inlineStr"/>
-      <c r="L367" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="368">
-      <c r="A368" s="4" t="inlineStr">
-        <is>
-          <t>12월 19일</t>
-        </is>
-      </c>
-      <c r="B368" s="4" t="inlineStr"/>
-      <c r="C368" s="4" t="inlineStr"/>
-      <c r="D368" s="4" t="inlineStr"/>
-      <c r="E368" s="4" t="inlineStr"/>
-      <c r="F368" s="4" t="inlineStr"/>
-      <c r="G368" s="4" t="inlineStr"/>
-      <c r="H368" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I368" s="4" t="inlineStr"/>
-      <c r="J368" s="4" t="inlineStr"/>
-      <c r="K368" s="4" t="inlineStr"/>
-      <c r="L368" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" s="4" t="inlineStr">
-        <is>
-          <t>12월 08일</t>
-        </is>
-      </c>
-      <c r="B369" s="4" t="inlineStr"/>
-      <c r="C369" s="4" t="inlineStr"/>
-      <c r="D369" s="4" t="inlineStr"/>
-      <c r="E369" s="4" t="inlineStr"/>
-      <c r="F369" s="4" t="inlineStr"/>
-      <c r="G369" s="4" t="inlineStr"/>
-      <c r="H369" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I369" s="4" t="inlineStr"/>
-      <c r="J369" s="4" t="inlineStr"/>
-      <c r="K369" s="4" t="inlineStr"/>
-      <c r="L369" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="370">
-      <c r="A370" s="4" t="inlineStr">
-        <is>
-          <t>11월 10일</t>
-        </is>
-      </c>
-      <c r="B370" s="4" t="inlineStr"/>
-      <c r="C370" s="4" t="inlineStr"/>
-      <c r="D370" s="4" t="inlineStr"/>
-      <c r="E370" s="4" t="inlineStr"/>
-      <c r="F370" s="4" t="inlineStr"/>
-      <c r="G370" s="4" t="inlineStr"/>
-      <c r="H370" s="4" t="inlineStr"/>
-      <c r="I370" s="4" t="inlineStr"/>
-      <c r="J370" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K370" s="4" t="inlineStr"/>
-      <c r="L370" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="371">
-      <c r="A371" s="4" t="inlineStr">
-        <is>
-          <t>11월 08일</t>
-        </is>
-      </c>
-      <c r="B371" s="4" t="inlineStr"/>
-      <c r="C371" s="4" t="inlineStr"/>
-      <c r="D371" s="4" t="inlineStr"/>
-      <c r="E371" s="4" t="inlineStr"/>
-      <c r="F371" s="4" t="inlineStr"/>
-      <c r="G371" s="4" t="inlineStr"/>
-      <c r="H371" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I371" s="4" t="inlineStr"/>
-      <c r="J371" s="4" t="inlineStr"/>
-      <c r="K371" s="4" t="inlineStr"/>
-      <c r="L371" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" s="4" t="inlineStr">
-        <is>
-          <t>10월 26일</t>
-        </is>
-      </c>
-      <c r="B372" s="4" t="inlineStr"/>
-      <c r="C372" s="4" t="inlineStr"/>
-      <c r="D372" s="4" t="inlineStr"/>
-      <c r="E372" s="4" t="inlineStr"/>
-      <c r="F372" s="4" t="inlineStr"/>
-      <c r="G372" s="4" t="inlineStr"/>
-      <c r="H372" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I372" s="4" t="inlineStr"/>
-      <c r="J372" s="4" t="inlineStr"/>
-      <c r="K372" s="4" t="inlineStr"/>
-      <c r="L372" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="373">
-      <c r="A373" s="4" t="inlineStr">
-        <is>
-          <t>10월 24일</t>
-        </is>
-      </c>
-      <c r="B373" s="4" t="inlineStr"/>
-      <c r="C373" s="4" t="inlineStr"/>
-      <c r="D373" s="4" t="inlineStr"/>
-      <c r="E373" s="4" t="inlineStr"/>
-      <c r="F373" s="4" t="inlineStr"/>
-      <c r="G373" s="4" t="inlineStr"/>
-      <c r="H373" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I373" s="4" t="inlineStr"/>
-      <c r="J373" s="4" t="inlineStr"/>
-      <c r="K373" s="4" t="inlineStr"/>
-      <c r="L373" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" s="4" t="inlineStr">
-        <is>
-          <t>10월 18일</t>
-        </is>
-      </c>
-      <c r="B374" s="4" t="inlineStr"/>
-      <c r="C374" s="4" t="inlineStr"/>
-      <c r="D374" s="4" t="inlineStr"/>
-      <c r="E374" s="4" t="inlineStr"/>
-      <c r="F374" s="4" t="inlineStr"/>
-      <c r="G374" s="4" t="inlineStr"/>
-      <c r="H374" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I374" s="4" t="inlineStr"/>
-      <c r="J374" s="4" t="inlineStr"/>
-      <c r="K374" s="4" t="inlineStr"/>
-      <c r="L374" s="5" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="375">
-      <c r="A375" s="4" t="inlineStr">
-        <is>
-          <t>10월 17일</t>
-        </is>
-      </c>
-      <c r="B375" s="4" t="inlineStr"/>
-      <c r="C375" s="4" t="inlineStr"/>
-      <c r="D375" s="4" t="inlineStr"/>
-      <c r="E375" s="4" t="inlineStr"/>
-      <c r="F375" s="4" t="inlineStr"/>
-      <c r="G375" s="4" t="inlineStr"/>
-      <c r="H375" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I375" s="4" t="inlineStr"/>
-      <c r="J375" s="4" t="inlineStr"/>
-      <c r="K375" s="4" t="inlineStr"/>
-      <c r="L375" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="376">
-      <c r="A376" s="4" t="inlineStr">
-        <is>
-          <t>10월 03일</t>
-        </is>
-      </c>
-      <c r="B376" s="4" t="inlineStr"/>
-      <c r="C376" s="4" t="inlineStr"/>
-      <c r="D376" s="4" t="inlineStr"/>
-      <c r="E376" s="4" t="inlineStr"/>
-      <c r="F376" s="4" t="inlineStr"/>
-      <c r="G376" s="4" t="inlineStr"/>
-      <c r="H376" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I376" s="4" t="inlineStr"/>
-      <c r="J376" s="4" t="inlineStr"/>
-      <c r="K376" s="4" t="inlineStr"/>
-      <c r="L376" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" s="4" t="inlineStr">
-        <is>
-          <t>09월 28일</t>
-        </is>
-      </c>
-      <c r="B377" s="4" t="inlineStr"/>
-      <c r="C377" s="4" t="inlineStr"/>
-      <c r="D377" s="4" t="inlineStr"/>
-      <c r="E377" s="4" t="inlineStr"/>
-      <c r="F377" s="4" t="inlineStr"/>
-      <c r="G377" s="4" t="inlineStr"/>
-      <c r="H377" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I377" s="4" t="inlineStr"/>
-      <c r="J377" s="4" t="inlineStr"/>
-      <c r="K377" s="4" t="inlineStr"/>
-      <c r="L377" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="378">
-      <c r="A378" s="4" t="inlineStr">
-        <is>
-          <t>09월 24일</t>
-        </is>
-      </c>
-      <c r="B378" s="4" t="inlineStr"/>
-      <c r="C378" s="4" t="inlineStr"/>
-      <c r="D378" s="4" t="inlineStr"/>
-      <c r="E378" s="4" t="inlineStr"/>
-      <c r="F378" s="4" t="inlineStr"/>
-      <c r="G378" s="4" t="inlineStr"/>
-      <c r="H378" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I378" s="4" t="inlineStr"/>
-      <c r="J378" s="4" t="inlineStr"/>
-      <c r="K378" s="4" t="inlineStr"/>
-      <c r="L378" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="379">
-      <c r="A379" s="4" t="inlineStr">
-        <is>
-          <t>09월 19일</t>
-        </is>
-      </c>
-      <c r="B379" s="4" t="inlineStr"/>
-      <c r="C379" s="4" t="inlineStr"/>
-      <c r="D379" s="4" t="inlineStr"/>
-      <c r="E379" s="4" t="inlineStr"/>
-      <c r="F379" s="4" t="inlineStr"/>
-      <c r="G379" s="4" t="inlineStr"/>
-      <c r="H379" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I379" s="4" t="inlineStr"/>
-      <c r="J379" s="4" t="inlineStr"/>
-      <c r="K379" s="4" t="inlineStr"/>
-      <c r="L379" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" s="4" t="inlineStr">
-        <is>
-          <t>09월 02일</t>
-        </is>
-      </c>
-      <c r="B380" s="4" t="inlineStr"/>
-      <c r="C380" s="4" t="inlineStr"/>
-      <c r="D380" s="4" t="inlineStr"/>
-      <c r="E380" s="4" t="inlineStr"/>
-      <c r="F380" s="4" t="inlineStr"/>
-      <c r="G380" s="4" t="inlineStr"/>
-      <c r="H380" s="4" t="inlineStr"/>
-      <c r="I380" s="4" t="inlineStr"/>
-      <c r="J380" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K380" s="4" t="inlineStr"/>
-      <c r="L380" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="381">
-      <c r="A381" s="4" t="inlineStr">
-        <is>
-          <t>06월 16일</t>
-        </is>
-      </c>
-      <c r="B381" s="4" t="inlineStr"/>
-      <c r="C381" s="4" t="inlineStr"/>
-      <c r="D381" s="4" t="inlineStr"/>
-      <c r="E381" s="4" t="inlineStr"/>
-      <c r="F381" s="4" t="inlineStr"/>
-      <c r="G381" s="4" t="inlineStr"/>
-      <c r="H381" s="4" t="inlineStr"/>
-      <c r="I381" s="4" t="inlineStr"/>
-      <c r="J381" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K381" s="4" t="inlineStr"/>
-      <c r="L381" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="382">
-      <c r="A382" s="4" t="inlineStr">
-        <is>
-          <t>11월 28일</t>
-        </is>
-      </c>
-      <c r="B382" s="4" t="inlineStr"/>
-      <c r="C382" s="4" t="inlineStr"/>
-      <c r="D382" s="4" t="inlineStr"/>
-      <c r="E382" s="4" t="inlineStr"/>
-      <c r="F382" s="4" t="inlineStr"/>
-      <c r="G382" s="4" t="inlineStr"/>
-      <c r="H382" s="4" t="inlineStr"/>
-      <c r="I382" s="4" t="inlineStr"/>
-      <c r="J382" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K382" s="4" t="inlineStr"/>
-      <c r="L382" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" s="4" t="inlineStr">
-        <is>
-          <t>11월 21일</t>
-        </is>
-      </c>
-      <c r="B383" s="4" t="inlineStr"/>
-      <c r="C383" s="4" t="inlineStr"/>
-      <c r="D383" s="4" t="inlineStr"/>
-      <c r="E383" s="4" t="inlineStr"/>
-      <c r="F383" s="4" t="inlineStr"/>
-      <c r="G383" s="4" t="inlineStr"/>
-      <c r="H383" s="4" t="inlineStr"/>
-      <c r="I383" s="4" t="inlineStr"/>
-      <c r="J383" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K383" s="4" t="inlineStr"/>
-      <c r="L383" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="384">
-      <c r="A384" s="4" t="inlineStr">
-        <is>
-          <t>11월 18일</t>
-        </is>
-      </c>
-      <c r="B384" s="4" t="inlineStr"/>
-      <c r="C384" s="4" t="inlineStr"/>
-      <c r="D384" s="4" t="inlineStr"/>
-      <c r="E384" s="4" t="inlineStr"/>
-      <c r="F384" s="4" t="inlineStr"/>
-      <c r="G384" s="4" t="inlineStr"/>
-      <c r="H384" s="4" t="inlineStr"/>
-      <c r="I384" s="4" t="inlineStr"/>
-      <c r="J384" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K384" s="4" t="inlineStr"/>
-      <c r="L384" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="385">
-      <c r="A385" s="4" t="inlineStr">
-        <is>
-          <t>11월 27일</t>
-        </is>
-      </c>
-      <c r="B385" s="4" t="inlineStr"/>
-      <c r="C385" s="4" t="inlineStr"/>
-      <c r="D385" s="4" t="inlineStr"/>
-      <c r="E385" s="4" t="inlineStr"/>
-      <c r="F385" s="4" t="inlineStr"/>
-      <c r="G385" s="4" t="inlineStr"/>
-      <c r="H385" s="4" t="inlineStr"/>
-      <c r="I385" s="4" t="inlineStr"/>
-      <c r="J385" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K385" s="4" t="inlineStr"/>
-      <c r="L385" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="386">
-      <c r="A386" s="4" t="inlineStr">
-        <is>
-          <t>02월 11일</t>
-        </is>
-      </c>
-      <c r="B386" s="4" t="inlineStr"/>
-      <c r="C386" s="4" t="inlineStr"/>
-      <c r="D386" s="4" t="inlineStr"/>
-      <c r="E386" s="4" t="inlineStr"/>
-      <c r="F386" s="4" t="inlineStr"/>
-      <c r="G386" s="4" t="inlineStr"/>
-      <c r="H386" s="4" t="inlineStr"/>
-      <c r="I386" s="4" t="inlineStr"/>
-      <c r="J386" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K386" s="4" t="inlineStr"/>
-      <c r="L386" s="5" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="387">
-      <c r="A387" s="6" t="inlineStr">
+      <c r="A353" s="6" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="B387" s="6" t="n">
-        <v>79</v>
-      </c>
-      <c r="C387" s="6" t="inlineStr"/>
-      <c r="D387" s="6" t="n">
+      <c r="B353" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="C353" s="6" t="inlineStr"/>
+      <c r="D353" s="6" t="n">
         <v>113</v>
       </c>
-      <c r="E387" s="6" t="inlineStr"/>
-      <c r="F387" s="6" t="n">
+      <c r="E353" s="6" t="inlineStr"/>
+      <c r="F353" s="6" t="n">
         <v>105</v>
       </c>
-      <c r="G387" s="6" t="inlineStr"/>
-      <c r="H387" s="6" t="n">
+      <c r="G353" s="6" t="inlineStr"/>
+      <c r="H353" s="6" t="n">
         <v>136</v>
       </c>
-      <c r="I387" s="6" t="n">
-        <v>43</v>
-      </c>
-      <c r="J387" s="6" t="n">
+      <c r="I353" s="6" t="inlineStr"/>
+      <c r="J353" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="K387" s="6" t="inlineStr"/>
-      <c r="L387" s="6" t="n">
-        <v>492</v>
+      <c r="K353" s="6" t="inlineStr"/>
+      <c r="L353" s="6" t="n">
+        <v>448</v>
       </c>
     </row>
   </sheetData>
@@ -9115,7 +8349,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>부정 리뷰 16건  |  그 중 신규 16건</t>
+          <t>부정 리뷰 16건  |  그 중 신규 0건</t>
         </is>
       </c>
     </row>
@@ -9569,7 +8803,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D84"/>
+  <dimension ref="A1:D83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -9595,7 +8829,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>부정 리뷰 79건  |  그 중 신규 79건</t>
+          <t>부정 리뷰 78건  |  그 중 신규 0건</t>
         </is>
       </c>
     </row>
@@ -11337,30 +10571,8 @@
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="8" t="inlineStr">
-        <is>
-          <t>06월 07일</t>
-        </is>
-      </c>
-      <c r="B84" s="9" t="inlineStr">
-        <is>
-          <t>Ryan Koo</t>
-        </is>
-      </c>
-      <c r="C84" s="10" t="inlineStr">
-        <is>
-          <t>1. 너무 많은 정보와 불필요한 디자인 요소로 데이터 잡아먹지 말고 저용량 트래픽 환경에서도 기본적인 거래에 어려움이 없도록 만들어주세요. 환경이 안좋을 때는 버벅임과 오류가 심해 주거래가 기업은행인데도 불편함 감수하고 케이뱅크로 해결했네요.. 2. 쿠팡이츠 연동 결재가 가끔 안되는데 오후 한시 반인데도.. 은행 점검서비스 시간이라고 거래가 안되네요. 어플 문제인가 싶어서 다른 은행 계좌로 했는데 진행에 어려움이 없었어요. 오후 1시 반에 점검으로 거래를 막지는 않았을테고 오류로 보여지는데 해결해주세요.</t>
-        </is>
-      </c>
-      <c r="D84" s="8" t="inlineStr">
-        <is>
-          <t>앱 실행/오류</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:D84"/>
+  <autoFilter ref="A5:D83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11461,7 +10673,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>부정 리뷰 113건  |  그 중 신규 113건</t>
+          <t>부정 리뷰 113건  |  그 중 신규 0건</t>
         </is>
       </c>
     </row>
@@ -14075,7 +13287,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>부정 리뷰 105건  |  그 중 신규 105건</t>
+          <t>부정 리뷰 105건  |  그 중 신규 0건</t>
         </is>
       </c>
     </row>
@@ -16513,7 +15725,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>부정 리뷰 136건  |  그 중 신규 136건</t>
+          <t>부정 리뷰 136건  |  그 중 신규 0건</t>
         </is>
       </c>
     </row>
@@ -19545,7 +18757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -19571,7 +18783,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>부정 리뷰 43건  |  그 중 신규 43건</t>
+          <t>수집된 부정 리뷰 없음</t>
         </is>
       </c>
     </row>
@@ -19597,978 +18809,8 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t>12월 17일</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>지이이이이영</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>[거꾸로 가는 앱 디자인] 그 전으로 다시 돌려주세여.........</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>디자인/사용성</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>01월 03일</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>ㅋㅇㅋㅁㅁㅇㅇ</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>[그냥 별로] 아이디도 제대로 못찾게 해놔서 개불편함ㅋㅋ</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>12월 06일</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>단거먹으면이아픔</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>[인류가만들어낸 쓰레기] 거지같네</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>11월 30일</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>승까</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>[이거뭐 인증도 안되고] 이거 쓰라고 만든앱이 아니라 열받으라고 만들었네
-은행을 바꿔야겠네 불편해서</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>11월 30일</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>거북스프</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>[왜 바꾼거냐] 그전에 쓰던 어플이 훨씬 보기좋고 편했는데 이따구로 만들어 놧네 심지어 거래내역은 버그땜에 확인도 안됨 왜 퇴보하냐;;;</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>앱 실행/오류</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>05월 12일</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>마오ㅛ어두터터어ㅓㅇ억ㄴ</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>[공인인증 타행 인증  다 와서  먹통이네요] 타행공인인증 기록 다  등록후  확인하려는데  확인 버튼 클릭이 안됩니다  수번  해봐도  안되요  보안카드 문제인가해서  교체했는데도  안됩니다  수정좀  해주세요 !ㅠ</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>앱 실행/오류</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>01월 25일</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>0개비</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>[Ars인증부터 오류가 납니다] 혹시나 전화차단목록에 있나 다 취소해보고도 해봤지만 그냥 이 앱 자체가 문제네요.
-기본적인 것도 안되면 어따 써먹어야 합니까?
-개발하고 직접 써보면 문제가 뭔지 아실텐데요?</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>앱 실행/오류</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>12월 30일</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>011.011</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>[로그인] 왜 로그인할때마다 장시간 사용이 어쩌구 하면서 끊기죠? 
-어짜피 다시로그인하는건데? 계속몇번을 그러네요 후</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>12월 17일</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>prkah</t>
-        </is>
-      </c>
-      <c r="C14" s="10" t="inlineStr">
-        <is>
-          <t>[Langauge change???] How to change in English langauge!!!</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>12월 14일</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>냉파스</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>[진짜 개안좋음] 진짜 이 어플 내가 쓰는 은행어플중 제일 겁나 최악이네요 리얼 되는거 하나없고 겁나 복잡하고 안되고 안눌리고 몇번을 인증하고 겁나 짜증나게 만드네요 여기 어플 진짜 최악입니다^^</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>디자인/사용성</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>11월 13일</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>메론레몬메론</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>[로그인창에서 멈춰서 로그인이 안됩니다] 로그인창에서 멈춰서 로그인이 안됩니다 
-오류 수정좀 해주세요 제발쫌</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>09월 25일</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>이불밖은-위험해</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>[타은행 앱을 한번도 이용해본적 없는 사람이 만든것같아요] 디자인도 너무 별로고 비밀번호 입력하면 저 멀리서도 보이게 아주 큰 폰트로 똭똭 입력돼서 참 황당하네요
-그리고 국민은행 어플쓰다가 이거쓰니까 너무 답답하고 하나 인증하니까 다른거 인증하라고 하고 에러나서 처음부터 다시하고... 이앱은 왜 만들었는지 사람 화나게 하려고 참을성 테스트하는 앱인가 싶어요</t>
-        </is>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>07월 04일</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>aylwtl</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>[아이폰 공인인증서 저장이안되네요] 정말 불편하네요. 공인인증서 로그인하려는데 저장도안되고</t>
-        </is>
-      </c>
-      <c r="D18" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>06월 14일</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>짱남 8272</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>[진짜 뭐같이 만들어놨네] 왜 기업은행이 다른 은행들보다 뒤처지고 평이 안좋은지 딱 알게 해두는 앱입니다. 최근 기업은행 카드 바꾼거 알림 문자에 누적 금액 이상하게 나와서 내역확인하려고 했더니 진짜 되는거 하나없고 인증만 몇번하고 기존 인증서는 폐지시키고... 신한은행 쏠의 반의반도 안되는 구린 어플이네요. 이 앱 담당자는 좀 직무유기 급이 아닌가 싶은데, 정신 좀 차리세요</t>
-        </is>
-      </c>
-      <c r="D19" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
-        <is>
-          <t>05월 09일</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>끄아아아아아아ㅏㅏ</t>
-        </is>
-      </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>[쓰라고 만든거 맞아요?] 로그인 지문인식해도 무슨 오류라고 계속 안들어가지고 어플 한번 들어가려면 몇번을 껐다켰다 해야하는건지 ㅋㅋ 쓰라고 만든거 맞아요? 타은행 뱅킹어플 대비 효율성 너무 떨어지고 잘 안쓰게됨</t>
-        </is>
-      </c>
-      <c r="D20" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
-        <is>
-          <t>12월 29일</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>내스스로</t>
-        </is>
-      </c>
-      <c r="C21" s="10" t="inlineStr">
-        <is>
-          <t>[이딴거 만들시간에] 똥이나 싸라죠</t>
-        </is>
-      </c>
-      <c r="D21" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>11월 07일</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>아니시를</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>[절대쓰지마요] 혈압올라서 못쓰겠네요</t>
-        </is>
-      </c>
-      <c r="D22" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>09월 02일</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>ㅎㅇㄷㄴㄹㅅㄱㅈ</t>
-        </is>
-      </c>
-      <c r="C23" s="10" t="inlineStr">
-        <is>
-          <t>[몇달전부터 앱 시작화면이 안뜨네요] 무한 로딩 아예 안되요 아이폰
-지우고 깔아도 똑같음</t>
-        </is>
-      </c>
-      <c r="D23" s="8" t="inlineStr">
-        <is>
-          <t>속도/성능</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>08월 16일</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Rinandhye</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>[이체 버튼을 계속 눌러도 반응이 없네요] 기업은행 앱 너무 불편합니다</t>
-        </is>
-      </c>
-      <c r="D24" s="8" t="inlineStr">
-        <is>
-          <t>이체/거래</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>08월 12일</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Juneeyah</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>[잘쓰던 휙송금 왜 없앤거죠...?] 이거 아님 켤일도 없는데 그걸 없애버리네요 하... 일부러 열받게 하려고 그러는건가</t>
-        </is>
-      </c>
-      <c r="D25" s="8" t="inlineStr">
-        <is>
-          <t>이체/거래</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>07월 14일</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>댓글거의안다는사람</t>
-        </is>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>[카드조회 하니까] 무슨 오류떴다고 다시시도 하라고 몇번이나 뜨네요
-은행가서 직접 발급받을랍니다</t>
-        </is>
-      </c>
-      <c r="D26" s="8" t="inlineStr">
-        <is>
-          <t>앱 실행/오류</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>07월 13일</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>먕근</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>[새로나온거못써서다시이거하려하는데] 공인인증서도안먹고ㅅㅂ
-새로나온거ㅈㄹ느리고조회도느리고짜증나는데
-이것때문에 카드도바꿔야하나
-카드바꾸면 가스전기 집요금 폰요금
-다기업은행연동했는데
-애초에기업은행카드ㅅㅂ만들지말껄ㅈ같네진짜</t>
-        </is>
-      </c>
-      <c r="D27" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>07월 12일</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>초밥마왕</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>[서비스] 아이디 찾기인데 아이디를 안알려주면 뭐어떻게 하라는겁니까  군인 입장에서 고객센터 상담도못하는데 진짜 심각하게 스트레스받네요</t>
-        </is>
-      </c>
-      <c r="D28" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>07월 11일</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Donghyul</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>[로그인 문제] 아니 간편번호 로그인 이용하던 사람인데 공인인증서 등록도 아직 안해놨는데 벌써 막아버리시면 안되죠 지금 계좌 잔액 확인도 못하고 애초에 미리 공지를 해놓으시면 인증서 등록 해놓았을텐데 황당하네요</t>
-        </is>
-      </c>
-      <c r="D29" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>07월 07일</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>던단</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>[최악의 어플] 별1개도 아깝다 쓰라고 만든건지 보일려고 만든건지 모르겠다 중국어플도 이보다 잘만들겠다 사용자체가 안되게 만들었다</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>06월 24일</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>BAMBOOMONSTER</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>[없어지나요 이것도] 뭔 갑자기 새로 어플받으라고...... 이것도 사라져요?</t>
-        </is>
-      </c>
-      <c r="D31" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>06월 10일</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>퀙</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>[천원 결제되었어요] 어떻게 된건가요? 취소해주세요!!</t>
-        </is>
-      </c>
-      <c r="D32" s="8" t="inlineStr">
-        <is>
-          <t>이체/거래</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>05월 04일</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>텐엑스</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>[페이스아이디] 어디로 사라짐?
-개선이라더니 퇴보하네....</t>
-        </is>
-      </c>
-      <c r="D33" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>04월 30일</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>Minqne</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>[페이스아이디 및 지문인식] 기능개선이라는데 페이스아이디 지문 인식 
-사라짐</t>
-        </is>
-      </c>
-      <c r="D34" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
-        <is>
-          <t>03월 12일</t>
-        </is>
-      </c>
-      <c r="B35" s="9" t="inlineStr">
-        <is>
-          <t>쟝이다요</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>[문의합니다] 타은행인증서등록하려고 들어가니ars인증하고나서 otp입력하고 다음단계로 넘어가는 버튼이안눌러져요 어플껐다켜도그렇고 핸드폰을다시 켜도그런데왜그런거죠? 은행이용을 못하고있어요ㅡㅡ 핸드폰산지 얼마되지않아서기계문제는아닌듯한데요</t>
-        </is>
-      </c>
-      <c r="D35" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>02월 27일</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>자운뎅</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>[타행기관 인증서 등록안되네요] 타행기관 인증서 등록안되네요
-이럴거면 모하러 만든건지....</t>
-        </is>
-      </c>
-      <c r="D36" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
-        <is>
-          <t>02월 24일</t>
-        </is>
-      </c>
-      <c r="B37" s="9" t="inlineStr">
-        <is>
-          <t>eishd</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>[공인인증서 등록이 안됩니다] 타행 발행 공인인증서 등록 화면에서 최종확인버튼이 눌리지 않습니다... 확인바랍니다 아이폰xr입니다</t>
-        </is>
-      </c>
-      <c r="D37" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>02월 06일</t>
-        </is>
-      </c>
-      <c r="B38" s="9" t="inlineStr">
-        <is>
-          <t>ㅎㅎ헿</t>
-        </is>
-      </c>
-      <c r="C38" s="10" t="inlineStr">
-        <is>
-          <t>[쓰라고 만든건지] 타행인증서 등록 왜 안해줘여 ㅋㅋㅋㅋㅋ 증는흐나</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>12월 02일</t>
-        </is>
-      </c>
-      <c r="B39" s="9" t="inlineStr">
-        <is>
-          <t>은행냄새</t>
-        </is>
-      </c>
-      <c r="C39" s="10" t="inlineStr">
-        <is>
-          <t>[One로그인] 아니 원로그인 아이디 찾으려고 아이디찾기에서 개인정보치고 들어가니까 아이디14개중에 앞에 3개 알려주면 어떡하라고</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>10월 23일</t>
-        </is>
-      </c>
-      <c r="B40" s="9" t="inlineStr">
-        <is>
-          <t>지뚱23</t>
-        </is>
-      </c>
-      <c r="C40" s="10" t="inlineStr">
-        <is>
-          <t>[아이폰x 이용자를 위한 안면인식] 안면인식 기능 빨리 넣어주세요 매번 공인인증서 암호 치기 귀찮아요 ㅠㅠ</t>
-        </is>
-      </c>
-      <c r="D40" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="8" t="inlineStr">
-        <is>
-          <t>10월 09일</t>
-        </is>
-      </c>
-      <c r="B41" s="9" t="inlineStr">
-        <is>
-          <t>ㄹㄹㄹㄹㄹㄹ쁄</t>
-        </is>
-      </c>
-      <c r="C41" s="10" t="inlineStr">
-        <is>
-          <t>[텆치가 안됨] 미니라고 해서 신나게 받았는데 결국 인증서 등록 과정 5번 하다가 빡쳐서 걍 일반어플 받아요ㅋ</t>
-        </is>
-      </c>
-      <c r="D41" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t>09월 30일</t>
-        </is>
-      </c>
-      <c r="B42" s="9" t="inlineStr">
-        <is>
-          <t>재미재미재미짐누엍</t>
-        </is>
-      </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>[지문 등록을 대체 몇번을 해야합니까] 분명 등록 해놓은 지문도 며칠 있으면 없다하네요
-5일에 한번은 지문을 재등록 하는데 진짜 이렇게 어플 만들거면 쓰지 말라는 거 아닌지</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t>인증/보안</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>08월 10일</t>
-        </is>
-      </c>
-      <c r="B43" s="9" t="inlineStr">
-        <is>
-          <t>기업은행전</t>
-        </is>
-      </c>
-      <c r="C43" s="10" t="inlineStr">
-        <is>
-          <t>[어플을 사용하란건지? 궁금하네요] 가입다하고등록다하고 나니깐 로그인자체가 안되고 
-아이폰이여서지문등록후 하는데 지문하는창도 뜨지도 않고 어플을 사용하라는건지아니면 다른어플을사용하라는건지 잘모르겠네요</t>
-        </is>
-      </c>
-      <c r="D43" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="8" t="inlineStr">
-        <is>
-          <t>08월 01일</t>
-        </is>
-      </c>
-      <c r="B44" s="9" t="inlineStr">
-        <is>
-          <t>ㅠ어댱ㅍ나덜</t>
-        </is>
-      </c>
-      <c r="C44" s="10" t="inlineStr">
-        <is>
-          <t>[아니 인증서는] 인증서를 타행거라고 복사를 안해주는거냐 어플이 먹통인거냐 무슨 은행업무를 시작도 못하게하네 장난하는것도 아니고 직원들한테 실적 올리라고 닥달하지말고 어플관리나 좀 잘해라</t>
-        </is>
-      </c>
-      <c r="D44" s="8" t="inlineStr">
-        <is>
-          <t>앱 실행/오류</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t>07월 27일</t>
-        </is>
-      </c>
-      <c r="B45" s="9" t="inlineStr">
-        <is>
-          <t>코멘트서치</t>
-        </is>
-      </c>
-      <c r="C45" s="10" t="inlineStr">
-        <is>
-          <t>[로그인할때 지문인식이 아예 뜨질 않습니다] 지문 재등록도 해보고 껐다 켜보기도했는데 지문인식 창이 뜨지도 않고 되지도 않아요</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t>로그인</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="8" t="inlineStr">
-        <is>
-          <t>07월 11일</t>
-        </is>
-      </c>
-      <c r="B46" s="9" t="inlineStr">
-        <is>
-          <t>Ming_블리</t>
-        </is>
-      </c>
-      <c r="C46" s="10" t="inlineStr">
-        <is>
-          <t>[구매목록삭제 부탁해요~] 구매목록삭제 부탁해요~</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="8" t="inlineStr">
-        <is>
-          <t>11월 20일</t>
-        </is>
-      </c>
-      <c r="B47" s="9" t="inlineStr">
-        <is>
-          <t>강탄소년단</t>
-        </is>
-      </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>[구매 목록 삭제 부탁드립니다] 구매 목록 삭제 부탁드립니다</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t>07월 31일</t>
-        </is>
-      </c>
-      <c r="B48" s="9" t="inlineStr">
-        <is>
-          <t>당근 돌아</t>
-        </is>
-      </c>
-      <c r="C48" s="10" t="inlineStr">
-        <is>
-          <t>[app이 자꾸 죽네.  아이폰까지 강제로 리부팅 시킴 ㅎㅎ] 얼마나 삼류 은행인지?
-은행가서 아이폰 6에서 자꾸 죽어서 아이폰 7로 바꾸고 사용하는데도.  앱이 실행후 앱이 없어지거나 아이폰이 리부팅됨. ㅎㅎ 대단해. ㅎㅎ 이런 게 학생 습작용이냐? 기업용이냐?
-우선, ibk 개인용 앱은 아주 잘 동작함. 앱이 튀기거나 리부팅 되는 경우가 없음 , 센터에 전화 하라고요?
-전화하니 사파리에서 캐쉬 지우고 새로 설치 하라고요? 다 해봄.  와이파이든 lte 든 5번 하면 한번 정고 성공함.  이게 앱인지? 
- 무능한게 아닌지? 
-특정 폰 문제? 위에 글쓴것 처럼 iphone 6/7 공통 현상임. 
-왜 개인용 앱은 잘되고?? 기업앱만 문제 일까요?</t>
-        </is>
-      </c>
-      <c r="D48" s="8" t="inlineStr">
-        <is>
-          <t>기타</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A5:D48"/>
+  <autoFilter ref="A5:D6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>